<commit_message>
Update: 2026-07-15 04:49 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AS$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AN$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AO$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1673,19 +1673,19 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1.050031252</v>
+        <v>1.050006898</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>5.25</v>
+        <v>5.38</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>33.4</v>
+        <v>30.1</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>12</v>
@@ -1704,7 +1704,8 @@
           <t>For v2:
 More hopstand and late hops
 Whc lax yeast
-Larger portion pilsener malt</t>
+Larger portion pilsener malt
+Used American Pale Ale water profile</t>
         </is>
       </c>
     </row>
@@ -1768,8 +1769,72 @@
       </c>
       <c r="P20" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>American IPA</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Jonas</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2019-03-08</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1.065578044</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>55.08</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Easy drink beer with tropical notes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P20"/>
+  <autoFilter ref="A1:P21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1780,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS74"/>
+  <dimension ref="A1:AT76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1828,6 +1893,7 @@
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
     <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2054,6 +2120,11 @@
       <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>notInRecipe</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>addAfterBoil</t>
         </is>
       </c>
     </row>
@@ -2160,6 +2231,7 @@
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2272,6 +2344,7 @@
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2378,6 +2451,7 @@
       <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2484,6 +2558,7 @@
       <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2590,6 +2665,7 @@
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2696,6 +2772,7 @@
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2829,6 +2906,7 @@
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2907,6 +2985,7 @@
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2985,6 +3064,7 @@
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3085,6 +3165,7 @@
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3163,6 +3244,7 @@
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3264,6 +3346,7 @@
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3391,6 +3474,7 @@
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3489,6 +3573,7 @@
       <c r="AQ15" t="inlineStr"/>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3598,6 +3683,7 @@
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3706,6 +3792,7 @@
       <c r="AQ17" t="inlineStr"/>
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3812,6 +3899,7 @@
       <c r="AQ18" t="inlineStr"/>
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3922,6 +4010,7 @@
       </c>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4023,6 +4112,7 @@
       <c r="AQ20" t="inlineStr"/>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4097,6 +4187,7 @@
       <c r="AQ21" t="inlineStr"/>
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4198,6 +4289,7 @@
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4325,6 +4417,7 @@
       <c r="AQ23" t="inlineStr"/>
       <c r="AR23" t="inlineStr"/>
       <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4403,6 +4496,7 @@
       <c r="AQ24" t="inlineStr"/>
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4481,6 +4575,7 @@
       <c r="AQ25" t="inlineStr"/>
       <c r="AR25" t="inlineStr"/>
       <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4608,6 +4703,7 @@
       <c r="AQ26" t="inlineStr"/>
       <c r="AR26" t="inlineStr"/>
       <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4741,6 +4837,7 @@
       <c r="AQ27" t="inlineStr"/>
       <c r="AR27" t="inlineStr"/>
       <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4849,6 +4946,7 @@
       </c>
       <c r="AR28" t="inlineStr"/>
       <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4955,6 +5053,7 @@
       <c r="AQ29" t="inlineStr"/>
       <c r="AR29" t="inlineStr"/>
       <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5033,6 +5132,7 @@
       <c r="AQ30" t="inlineStr"/>
       <c r="AR30" t="inlineStr"/>
       <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5139,6 +5239,7 @@
       <c r="AQ31" t="inlineStr"/>
       <c r="AR31" t="inlineStr"/>
       <c r="AS31" t="inlineStr"/>
+      <c r="AT31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5217,6 +5318,7 @@
       <c r="AQ32" t="inlineStr"/>
       <c r="AR32" t="inlineStr"/>
       <c r="AS32" t="inlineStr"/>
+      <c r="AT32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5318,6 +5420,7 @@
       <c r="AQ33" t="inlineStr"/>
       <c r="AR33" t="inlineStr"/>
       <c r="AS33" t="inlineStr"/>
+      <c r="AT33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5439,6 +5542,7 @@
       <c r="AQ34" t="inlineStr"/>
       <c r="AR34" t="inlineStr"/>
       <c r="AS34" t="inlineStr"/>
+      <c r="AT34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5540,6 +5644,7 @@
       <c r="AQ35" t="inlineStr"/>
       <c r="AR35" t="inlineStr"/>
       <c r="AS35" t="inlineStr"/>
+      <c r="AT35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5646,6 +5751,7 @@
       <c r="AQ36" t="inlineStr"/>
       <c r="AR36" t="inlineStr"/>
       <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5774,6 +5880,7 @@
       <c r="AQ37" t="inlineStr"/>
       <c r="AR37" t="inlineStr"/>
       <c r="AS37" t="inlineStr"/>
+      <c r="AT37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5877,6 +5984,7 @@
       </c>
       <c r="AR38" t="inlineStr"/>
       <c r="AS38" t="inlineStr"/>
+      <c r="AT38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5982,6 +6090,7 @@
       <c r="AQ39" t="inlineStr"/>
       <c r="AR39" t="inlineStr"/>
       <c r="AS39" t="inlineStr"/>
+      <c r="AT39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6111,6 +6220,7 @@
       </c>
       <c r="AR40" t="inlineStr"/>
       <c r="AS40" t="inlineStr"/>
+      <c r="AT40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6240,6 +6350,7 @@
         <v>1</v>
       </c>
       <c r="AS41" t="inlineStr"/>
+      <c r="AT41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6344,6 +6455,7 @@
       <c r="AQ42" t="inlineStr"/>
       <c r="AR42" t="inlineStr"/>
       <c r="AS42" t="inlineStr"/>
+      <c r="AT42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6456,6 +6568,7 @@
       <c r="AQ43" t="inlineStr"/>
       <c r="AR43" t="inlineStr"/>
       <c r="AS43" t="inlineStr"/>
+      <c r="AT43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6530,6 +6643,7 @@
       <c r="AQ44" t="inlineStr"/>
       <c r="AR44" t="inlineStr"/>
       <c r="AS44" t="inlineStr"/>
+      <c r="AT44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6648,6 +6762,7 @@
       </c>
       <c r="AR45" t="inlineStr"/>
       <c r="AS45" t="inlineStr"/>
+      <c r="AT45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6760,6 +6875,7 @@
       <c r="AQ46" t="inlineStr"/>
       <c r="AR46" t="inlineStr"/>
       <c r="AS46" t="inlineStr"/>
+      <c r="AT46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6868,6 +6984,7 @@
       <c r="AQ47" t="inlineStr"/>
       <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr"/>
+      <c r="AT47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6969,6 +7086,7 @@
       <c r="AQ48" t="inlineStr"/>
       <c r="AR48" t="inlineStr"/>
       <c r="AS48" t="inlineStr"/>
+      <c r="AT48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7096,6 +7214,7 @@
       <c r="AQ49" t="inlineStr"/>
       <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr"/>
+      <c r="AT49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7208,6 +7327,7 @@
       <c r="AQ50" t="inlineStr"/>
       <c r="AR50" t="inlineStr"/>
       <c r="AS50" t="inlineStr"/>
+      <c r="AT50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7314,6 +7434,7 @@
       <c r="AQ51" t="inlineStr"/>
       <c r="AR51" t="inlineStr"/>
       <c r="AS51" t="inlineStr"/>
+      <c r="AT51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7392,6 +7513,7 @@
       <c r="AQ52" t="inlineStr"/>
       <c r="AR52" t="inlineStr"/>
       <c r="AS52" t="inlineStr"/>
+      <c r="AT52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7470,6 +7592,7 @@
       <c r="AQ53" t="inlineStr"/>
       <c r="AR53" t="inlineStr"/>
       <c r="AS53" t="inlineStr"/>
+      <c r="AT53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7570,6 +7693,7 @@
       <c r="AQ54" t="inlineStr"/>
       <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
+      <c r="AT54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7685,6 +7809,7 @@
       <c r="AQ55" t="inlineStr"/>
       <c r="AR55" t="inlineStr"/>
       <c r="AS55" t="inlineStr"/>
+      <c r="AT55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7786,6 +7911,7 @@
       <c r="AS56" t="b">
         <v>0</v>
       </c>
+      <c r="AT56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7894,6 +8020,7 @@
       </c>
       <c r="AR57" t="inlineStr"/>
       <c r="AS57" t="inlineStr"/>
+      <c r="AT57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8002,6 +8129,7 @@
       <c r="AQ58" t="inlineStr"/>
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
+      <c r="AT58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8111,6 +8239,7 @@
       </c>
       <c r="AR59" t="inlineStr"/>
       <c r="AS59" t="inlineStr"/>
+      <c r="AT59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8189,6 +8318,7 @@
       <c r="AQ60" t="inlineStr"/>
       <c r="AR60" t="inlineStr"/>
       <c r="AS60" t="inlineStr"/>
+      <c r="AT60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8267,6 +8397,7 @@
       <c r="AQ61" t="inlineStr"/>
       <c r="AR61" t="inlineStr"/>
       <c r="AS61" t="inlineStr"/>
+      <c r="AT61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8367,6 +8498,7 @@
       <c r="AQ62" t="inlineStr"/>
       <c r="AR62" t="inlineStr"/>
       <c r="AS62" t="inlineStr"/>
+      <c r="AT62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8475,6 +8607,7 @@
       </c>
       <c r="AR63" t="inlineStr"/>
       <c r="AS63" t="inlineStr"/>
+      <c r="AT63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8578,6 +8711,7 @@
         <v>0</v>
       </c>
       <c r="AS64" t="inlineStr"/>
+      <c r="AT64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8679,6 +8813,7 @@
       <c r="AQ65" t="inlineStr"/>
       <c r="AR65" t="inlineStr"/>
       <c r="AS65" t="inlineStr"/>
+      <c r="AT65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8800,6 +8935,7 @@
       <c r="AQ66" t="inlineStr"/>
       <c r="AR66" t="inlineStr"/>
       <c r="AS66" t="inlineStr"/>
+      <c r="AT66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8905,6 +9041,7 @@
       <c r="AQ67" t="inlineStr"/>
       <c r="AR67" t="inlineStr"/>
       <c r="AS67" t="inlineStr"/>
+      <c r="AT67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8924,98 +9061,71 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 207000000, "_seconds": 1776345941}</t>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>default-0aa30343c0c</t>
+          <t>default-c3ff8bb88f9</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>7MQ6Noi2PwgQW8SivnCh6TS5Y4oFMA</t>
+          <t>tqtVycoLMiKmJMplyu7GCIAsAeeETL</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 50000000, "_seconds": 1777108187}</t>
+          <t>{"_nanoseconds": 476000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>1777108187050</v>
+        <v>1781339591476</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>3.0.0</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="L68" t="n">
-        <v>2</v>
-      </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="P68" t="n">
-        <v>1</v>
+        <v>2.45</v>
       </c>
       <c r="Q68" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="S68" t="n">
-        <v>76</v>
-      </c>
-      <c r="U68" t="n">
-        <v>81</v>
-      </c>
-      <c r="V68" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Base (Pilsner)</t>
+        </is>
+      </c>
+      <c r="X68" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>Swaen Pilsner</t>
+        </is>
+      </c>
+      <c r="AE68" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF68" t="inlineStr"/>
+      <c r="AG68" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH68" t="n">
+        <v>74.23999999999999</v>
+      </c>
+      <c r="AI68" t="n">
+        <v>1.0368</v>
+      </c>
+      <c r="AJ68" t="n">
         <v>80</v>
-      </c>
-      <c r="W68" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="X68" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y68" t="inlineStr"/>
-      <c r="Z68" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="AB68" t="n">
-        <v>100</v>
-      </c>
-      <c r="AC68" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="AD68" t="inlineStr">
-        <is>
-          <t>Swaen Ale</t>
-        </is>
-      </c>
-      <c r="AE68" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF68" t="inlineStr">
-        <is>
-          <t>Swaen Ale is used to correct over-pale malts, to produce "golden" beer and to improve palate fullness.</t>
-        </is>
-      </c>
-      <c r="AG68" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="AH68" t="n">
-        <v>61.16</v>
-      </c>
-      <c r="AI68" t="n">
-        <v>1.037</v>
-      </c>
-      <c r="AJ68" t="n">
-        <v>80.13</v>
-      </c>
-      <c r="AK68" t="n">
-        <v>11.5</v>
       </c>
       <c r="AL68" t="inlineStr"/>
       <c r="AM68" t="inlineStr">
@@ -9033,6 +9143,7 @@
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
       <c r="AS68" t="inlineStr"/>
+      <c r="AT68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9052,52 +9163,52 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>default-c3ff8bb88f9</t>
+          <t>default-d9e04639a2c</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>dVHriCxcQvFiRnK1pq8TNs8Aop6maI</t>
+          <t>zNojkfDZoro1z7t7fMQtUDJKvZGT6s</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 684000000, "_seconds": 1777108192}</t>
+          <t>{"_nanoseconds": 852000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1777108192684</v>
+        <v>1781339591852</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>3.0.0</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="L69" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="Q69" t="n">
-        <v>1.9</v>
+        <v>5.1</v>
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>Base (Pilsner)</t>
+          <t>Base (Vienna)</t>
         </is>
       </c>
       <c r="X69" t="b">
         <v>0</v>
       </c>
       <c r="Z69" t="n">
-        <v>7.8</v>
+        <v>2.85</v>
       </c>
       <c r="AD69" t="inlineStr">
         <is>
-          <t>Swaen Pilsner</t>
+          <t>Swaen Vienna</t>
         </is>
       </c>
       <c r="AE69" t="b">
@@ -9110,13 +9221,13 @@
         </is>
       </c>
       <c r="AH69" t="n">
-        <v>36.7</v>
+        <v>15.15</v>
       </c>
       <c r="AI69" t="n">
-        <v>1.0368</v>
+        <v>1.03588</v>
       </c>
       <c r="AJ69" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AL69" t="inlineStr"/>
       <c r="AM69" t="inlineStr">
@@ -9132,10 +9243,9 @@
       <c r="AO69" t="inlineStr"/>
       <c r="AP69" t="inlineStr"/>
       <c r="AQ69" t="inlineStr"/>
-      <c r="AR69" t="b">
-        <v>0</v>
-      </c>
+      <c r="AR69" t="inlineStr"/>
       <c r="AS69" t="inlineStr"/>
+      <c r="AT69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9155,75 +9265,91 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>default-25ba5c7007d</t>
+          <t>default-c454dca637a</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>rvKpzQzk7zcFyo8SUDwJClJQhEMsUP</t>
+          <t>wqxhntH7cVkHGBGQHdmwHvGQQ8QOhy</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 305000000, "_seconds": 1776345994}</t>
+          <t>{"_nanoseconds": 50000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>1776345994305</v>
+        <v>1781339591050</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>3.0.0</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="L70" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.3</v>
+      </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="P70" t="n">
+        <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>61</v>
+        <v>6.6</v>
+      </c>
+      <c r="S70" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="U70" t="n">
+        <v>80</v>
+      </c>
+      <c r="V70" t="n">
+        <v>80</v>
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>Crystal/Caramel</t>
+          <t>Base (Munich)</t>
         </is>
       </c>
       <c r="X70" t="b">
         <v>0</v>
       </c>
+      <c r="Y70" t="inlineStr"/>
       <c r="Z70" t="n">
-        <v>2</v>
+        <v>2.54</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>4.6</v>
       </c>
       <c r="AD70" t="inlineStr">
         <is>
-          <t>GoldSwaen Classic</t>
+          <t>Swaen Munich Light</t>
         </is>
       </c>
       <c r="AE70" t="b">
         <v>0</v>
       </c>
-      <c r="AF70" t="inlineStr">
-        <is>
-          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
-        </is>
-      </c>
+      <c r="AF70" t="inlineStr"/>
       <c r="AG70" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
       <c r="AH70" t="n">
-        <v>2.14</v>
+        <v>9.09</v>
       </c>
       <c r="AI70" t="n">
-        <v>1.034</v>
+        <v>1.035</v>
       </c>
       <c r="AJ70" t="n">
-        <v>73.9130435</v>
+        <v>75.37</v>
+      </c>
+      <c r="AK70" t="n">
+        <v>11.7</v>
       </c>
       <c r="AL70" t="inlineStr"/>
       <c r="AM70" t="inlineStr">
@@ -9241,16 +9367,17 @@
       <c r="AQ70" t="inlineStr"/>
       <c r="AR70" t="inlineStr"/>
       <c r="AS70" t="inlineStr"/>
+      <c r="AT70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+          <t>yiPSN3Y6mmATMzlZ26e4uWlmbGRxaD</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>First lager</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -9258,52 +9385,54 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>default-HM41QfsZjsnkL2GS5s3sTYkVX5OKSM</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="n">
-        <v>0</v>
+          <t>default-25ba5c7007d</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>lBdAIVmlcp7FjYPSV55HleXloB6alW</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 491000000, "_seconds": 1781339589}</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>1781339589491</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
       </c>
       <c r="L71" t="n">
-        <v>3</v>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="P71" t="n">
-        <v>1.5</v>
+        <v>0.05</v>
       </c>
       <c r="Q71" t="n">
-        <v>1.8527919</v>
-      </c>
-      <c r="S71" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Crystal/Caramel</t>
         </is>
       </c>
       <c r="X71" t="b">
         <v>0</v>
       </c>
-      <c r="Y71" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB71" t="n">
-        <v>100</v>
-      </c>
-      <c r="AC71" t="n">
-        <v>4.5</v>
+      <c r="Z71" t="n">
+        <v>1.36</v>
       </c>
       <c r="AD71" t="inlineStr">
         <is>
-          <t>Clear Choice Malt ® Extra Pale</t>
+          <t>GoldSwaen Classic</t>
         </is>
       </c>
       <c r="AE71" t="b">
@@ -9311,30 +9440,27 @@
       </c>
       <c r="AF71" t="inlineStr">
         <is>
-          <t>Clear Choice Malt ® does not contain polyphenols thus reducing the risk of haze formation, increasing shelf life and reducing cold conditioning costs</t>
+          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
         </is>
       </c>
       <c r="AG71" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="AH71" t="n">
-        <v>68.18000000000001</v>
+        <v>1.52</v>
       </c>
       <c r="AI71" t="n">
-        <v>1.038</v>
+        <v>1.034</v>
       </c>
       <c r="AJ71" t="n">
-        <v>81.5</v>
-      </c>
-      <c r="AK71" t="n">
-        <v>10.1</v>
+        <v>73.9130435</v>
       </c>
       <c r="AL71" t="inlineStr"/>
       <c r="AM71" t="inlineStr">
         <is>
-          <t>Crisp</t>
+          <t>The Swaen</t>
         </is>
       </c>
       <c r="AN71" t="inlineStr">
@@ -9347,6 +9473,7 @@
       <c r="AQ71" t="inlineStr"/>
       <c r="AR71" t="inlineStr"/>
       <c r="AS71" t="inlineStr"/>
+      <c r="AT71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9367,7 +9494,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>default-x1sQkldAFEgNTfYCHtBq70SjihT1F8</t>
+          <t>default-HM41QfsZjsnkL2GS5s3sTYkVX5OKSM</t>
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
@@ -9378,21 +9505,21 @@
         <v>0</v>
       </c>
       <c r="L72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M72" t="inlineStr"/>
       <c r="P72" t="n">
         <v>1.5</v>
       </c>
       <c r="Q72" t="n">
-        <v>3.9593909</v>
+        <v>1.8527919</v>
       </c>
       <c r="S72" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>Base (Vienna)</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="X72" t="b">
@@ -9409,7 +9536,7 @@
       </c>
       <c r="AD72" t="inlineStr">
         <is>
-          <t>Vienna Malt</t>
+          <t>Clear Choice Malt ® Extra Pale</t>
         </is>
       </c>
       <c r="AE72" t="b">
@@ -9417,7 +9544,7 @@
       </c>
       <c r="AF72" t="inlineStr">
         <is>
-          <t>Vienna malt is produced on a conventional kiln and provides a light golden hue</t>
+          <t>Clear Choice Malt ® does not contain polyphenols thus reducing the risk of haze formation, increasing shelf life and reducing cold conditioning costs</t>
         </is>
       </c>
       <c r="AG72" t="inlineStr">
@@ -9426,16 +9553,16 @@
         </is>
       </c>
       <c r="AH72" t="n">
-        <v>22.73</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="AI72" t="n">
-        <v>1.037</v>
+        <v>1.038</v>
       </c>
       <c r="AJ72" t="n">
-        <v>80</v>
+        <v>81.5</v>
       </c>
       <c r="AK72" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="AL72" t="inlineStr"/>
       <c r="AM72" t="inlineStr">
@@ -9453,6 +9580,7 @@
       <c r="AQ72" t="inlineStr"/>
       <c r="AR72" t="inlineStr"/>
       <c r="AS72" t="inlineStr"/>
+      <c r="AT72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9470,75 +9598,83 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>default-sabmjufsad</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>TbX832JbWp5BHVi5ATe4AaXk3nMfr9</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
-        </is>
-      </c>
-      <c r="I73" t="n">
-        <v>1706434202728</v>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>2.10.5</t>
-        </is>
+          <t>default-x1sQkldAFEgNTfYCHtBq70SjihT1F8</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="n">
+        <v>0</v>
       </c>
       <c r="L73" t="n">
-        <v>0.3</v>
+        <v>1</v>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="P73" t="n">
+        <v>1.5</v>
       </c>
       <c r="Q73" t="n">
-        <v>2</v>
+        <v>3.9593909</v>
+      </c>
+      <c r="S73" t="n">
+        <v>50</v>
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Base (Vienna)</t>
         </is>
       </c>
       <c r="X73" t="b">
         <v>0</v>
       </c>
-      <c r="Z73" t="n">
-        <v>-2.29</v>
+      <c r="Y73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>4.5</v>
       </c>
       <c r="AD73" t="inlineStr">
         <is>
-          <t>Pale Malt 2-Row</t>
+          <t>Vienna Malt</t>
         </is>
       </c>
       <c r="AE73" t="b">
         <v>0</v>
       </c>
-      <c r="AF73" t="inlineStr"/>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>Vienna malt is produced on a conventional kiln and provides a light golden hue</t>
+        </is>
+      </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="AH73" t="n">
-        <v>6.82</v>
+        <v>22.73</v>
       </c>
       <c r="AI73" t="n">
-        <v>1.036</v>
+        <v>1.037</v>
+      </c>
+      <c r="AJ73" t="n">
+        <v>80</v>
+      </c>
+      <c r="AK73" t="n">
+        <v>9.6</v>
       </c>
       <c r="AL73" t="inlineStr"/>
       <c r="AM73" t="inlineStr">
         <is>
-          <t>SAB</t>
+          <t>Crisp</t>
         </is>
       </c>
       <c r="AN73" t="inlineStr">
@@ -9549,10 +9685,9 @@
       <c r="AO73" t="inlineStr"/>
       <c r="AP73" t="inlineStr"/>
       <c r="AQ73" t="inlineStr"/>
-      <c r="AR73" t="b">
-        <v>0</v>
-      </c>
+      <c r="AR73" t="inlineStr"/>
       <c r="AS73" t="inlineStr"/>
+      <c r="AT73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9572,108 +9707,73 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 526000000, "_seconds": 1706434203}</t>
+          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>default-4c1345c</t>
+          <t>default-sabmjufsad</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KAv9WQAuhq3uEgowTzBf8YrHtXE4LO</t>
+          <t>TbX832JbWp5BHVi5ATe4AaXk3nMfr9</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 140000000, "_seconds": 1712314604}</t>
+          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
         </is>
       </c>
       <c r="I74" t="n">
-        <v>1712314604140</v>
+        <v>1706434202728</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2.10.6</t>
-        </is>
-      </c>
-      <c r="K74" t="n">
+          <t>2.10.5</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q74" t="n">
         <v>2</v>
       </c>
-      <c r="L74" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M74" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="P74" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Q74" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="S74" t="n">
-        <v>0</v>
-      </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>Acidulated</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="X74" t="b">
         <v>0</v>
       </c>
-      <c r="Y74" t="n">
-        <v>0</v>
-      </c>
       <c r="Z74" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="AB74" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC74" t="n">
-        <v>4</v>
+        <v>-2.29</v>
       </c>
       <c r="AD74" t="inlineStr">
         <is>
-          <t>Acidulated</t>
+          <t>Pale Malt 2-Row</t>
         </is>
       </c>
       <c r="AE74" t="b">
         <v>0</v>
       </c>
-      <c r="AF74" t="inlineStr">
-        <is>
-          <t>Used in Germany to lower PH levels without resorting to chemicals. Lowers mash pH levels, lightens color, improves flavor stability.</t>
-        </is>
-      </c>
+      <c r="AF74" t="inlineStr"/>
       <c r="AG74" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="AH74" t="n">
-        <v>2.27</v>
+        <v>6.82</v>
       </c>
       <c r="AI74" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AJ74" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="AK74" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL74" t="inlineStr">
-        <is>
-          <t>Pale Liquid Extract</t>
-        </is>
-      </c>
+        <v>1.036</v>
+      </c>
+      <c r="AL74" t="inlineStr"/>
       <c r="AM74" t="inlineStr">
         <is>
-          <t>Weyermann</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="AN74" t="inlineStr">
@@ -9684,11 +9784,245 @@
       <c r="AO74" t="inlineStr"/>
       <c r="AP74" t="inlineStr"/>
       <c r="AQ74" t="inlineStr"/>
-      <c r="AR74" t="inlineStr"/>
+      <c r="AR74" t="b">
+        <v>0</v>
+      </c>
       <c r="AS74" t="inlineStr"/>
+      <c r="AT74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>First lager</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 526000000, "_seconds": 1706434203}</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>default-4c1345c</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>KAv9WQAuhq3uEgowTzBf8YrHtXE4LO</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 140000000, "_seconds": 1712314604}</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>1712314604140</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K75" t="n">
+        <v>2</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="P75" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="S75" t="n">
+        <v>0</v>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Acidulated</t>
+        </is>
+      </c>
+      <c r="X75" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>Acidulated</t>
+        </is>
+      </c>
+      <c r="AE75" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>Used in Germany to lower PH levels without resorting to chemicals. Lowers mash pH levels, lightens color, improves flavor stability.</t>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="AH75" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="AI75" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AJ75" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="AK75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL75" t="inlineStr">
+        <is>
+          <t>Pale Liquid Extract</t>
+        </is>
+      </c>
+      <c r="AM75" t="inlineStr">
+        <is>
+          <t>Weyermann</t>
+        </is>
+      </c>
+      <c r="AN75" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO75" t="inlineStr"/>
+      <c r="AP75" t="inlineStr"/>
+      <c r="AQ75" t="inlineStr"/>
+      <c r="AR75" t="inlineStr"/>
+      <c r="AS75" t="inlineStr"/>
+      <c r="AT75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>new-eNDTHs2wb879roS3Dq1orvcb3ATgbD</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="n">
+        <v>13.18</v>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="n">
+        <v>3</v>
+      </c>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="inlineStr"/>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Base (Maris Otter)</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr"/>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr"/>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>Pale Malt, Maris Otter</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AF76" t="inlineStr"/>
+      <c r="AG76" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH76" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI76" t="n">
+        <v>1.03795</v>
+      </c>
+      <c r="AJ76" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="AK76" t="inlineStr"/>
+      <c r="AL76" t="inlineStr"/>
+      <c r="AM76" t="inlineStr">
+        <is>
+          <t>Maris Otter</t>
+        </is>
+      </c>
+      <c r="AN76" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO76" t="inlineStr"/>
+      <c r="AP76" t="inlineStr"/>
+      <c r="AQ76" t="inlineStr"/>
+      <c r="AR76" t="inlineStr"/>
+      <c r="AS76" t="inlineStr"/>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AS74"/>
+  <autoFilter ref="A1:AT76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9699,7 +10033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN60"/>
+  <dimension ref="A1:AO64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9707,7 +10041,7 @@
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
@@ -9742,6 +10076,7 @@
     <col width="11" customWidth="1" min="38" max="38"/>
     <col width="10" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
+    <col width="11" customWidth="1" min="41" max="41"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9943,6 +10278,11 @@
       <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>day</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>_editFlag</t>
         </is>
       </c>
     </row>
@@ -10029,6 +10369,7 @@
       <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10133,6 +10474,7 @@
       </c>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10217,6 +10559,7 @@
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10301,6 +10644,7 @@
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10373,6 +10717,7 @@
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10445,6 +10790,7 @@
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10539,6 +10885,7 @@
       </c>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10633,6 +10980,7 @@
       </c>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10727,6 +11075,7 @@
       </c>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10835,6 +11184,7 @@
       </c>
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10943,6 +11293,7 @@
       </c>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11051,6 +11402,7 @@
       </c>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11159,6 +11511,7 @@
       </c>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -11267,6 +11620,7 @@
       </c>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11371,6 +11725,7 @@
       </c>
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11478,6 +11833,7 @@
       </c>
       <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11572,6 +11928,7 @@
       </c>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -11656,6 +12013,7 @@
       <c r="AL19" t="inlineStr"/>
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11764,6 +12122,7 @@
       </c>
       <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11872,6 +12231,7 @@
       </c>
       <c r="AM21" t="inlineStr"/>
       <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11980,6 +12340,7 @@
       </c>
       <c r="AM22" t="inlineStr"/>
       <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12088,6 +12449,7 @@
       </c>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -12172,6 +12534,7 @@
       <c r="AL24" t="inlineStr"/>
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12266,6 +12629,7 @@
       </c>
       <c r="AM25" t="inlineStr"/>
       <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -12373,6 +12737,7 @@
       </c>
       <c r="AM26" t="inlineStr"/>
       <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -12481,6 +12846,7 @@
       </c>
       <c r="AM27" t="inlineStr"/>
       <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12589,6 +12955,7 @@
       </c>
       <c r="AM28" t="inlineStr"/>
       <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -12697,6 +13064,7 @@
       </c>
       <c r="AM29" t="inlineStr"/>
       <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -12791,6 +13159,7 @@
       </c>
       <c r="AM30" t="inlineStr"/>
       <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12885,6 +13254,7 @@
       </c>
       <c r="AM31" t="inlineStr"/>
       <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -12992,6 +13362,7 @@
         <v>0</v>
       </c>
       <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13096,6 +13467,7 @@
       </c>
       <c r="AM33" t="inlineStr"/>
       <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13204,6 +13576,7 @@
       </c>
       <c r="AM34" t="inlineStr"/>
       <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -13316,6 +13689,7 @@
       <c r="AN35" t="n">
         <v>4</v>
       </c>
+      <c r="AO35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -13424,6 +13798,7 @@
       <c r="AN36" t="n">
         <v>4</v>
       </c>
+      <c r="AO36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -13508,6 +13883,7 @@
       <c r="AL37" t="inlineStr"/>
       <c r="AM37" t="inlineStr"/>
       <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -13616,6 +13992,7 @@
       </c>
       <c r="AM38" t="inlineStr"/>
       <c r="AN38" t="inlineStr"/>
+      <c r="AO38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -13710,6 +14087,7 @@
       </c>
       <c r="AM39" t="inlineStr"/>
       <c r="AN39" t="inlineStr"/>
+      <c r="AO39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -13804,6 +14182,7 @@
       </c>
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" t="inlineStr"/>
+      <c r="AO40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -13900,6 +14279,7 @@
       <c r="AL41" t="inlineStr"/>
       <c r="AM41" t="inlineStr"/>
       <c r="AN41" t="inlineStr"/>
+      <c r="AO41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -13994,6 +14374,7 @@
       </c>
       <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14087,6 +14468,7 @@
         <v>-100</v>
       </c>
       <c r="AN43" t="inlineStr"/>
+      <c r="AO43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14159,6 +14541,7 @@
       <c r="AL44" t="inlineStr"/>
       <c r="AM44" t="inlineStr"/>
       <c r="AN44" t="inlineStr"/>
+      <c r="AO44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14253,6 +14636,7 @@
       </c>
       <c r="AM45" t="inlineStr"/>
       <c r="AN45" t="inlineStr"/>
+      <c r="AO45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14360,6 +14744,7 @@
       </c>
       <c r="AM46" t="inlineStr"/>
       <c r="AN46" t="inlineStr"/>
+      <c r="AO46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14432,6 +14817,7 @@
       <c r="AL47" t="inlineStr"/>
       <c r="AM47" t="inlineStr"/>
       <c r="AN47" t="inlineStr"/>
+      <c r="AO47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14539,6 +14925,7 @@
       </c>
       <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
+      <c r="AO48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -14636,6 +15023,7 @@
       </c>
       <c r="AM49" t="inlineStr"/>
       <c r="AN49" t="inlineStr"/>
+      <c r="AO49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -14708,6 +15096,7 @@
       <c r="AL50" t="inlineStr"/>
       <c r="AM50" t="inlineStr"/>
       <c r="AN50" t="inlineStr"/>
+      <c r="AO50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -14782,6 +15171,7 @@
       <c r="AK51" t="inlineStr"/>
       <c r="AL51" t="inlineStr"/>
       <c r="AN51" t="inlineStr"/>
+      <c r="AO51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -14856,6 +15246,7 @@
       <c r="AK52" t="inlineStr"/>
       <c r="AL52" t="inlineStr"/>
       <c r="AN52" t="inlineStr"/>
+      <c r="AO52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -14882,7 +15273,7 @@
         <v>6.3</v>
       </c>
       <c r="H53" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J53" t="n">
         <v>3.5</v>
@@ -14894,7 +15285,7 @@
         <v>30</v>
       </c>
       <c r="Q53" t="n">
-        <v>16.1</v>
+        <v>15</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -14963,6 +15354,7 @@
       </c>
       <c r="AM53" t="inlineStr"/>
       <c r="AN53" t="inlineStr"/>
+      <c r="AO53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -14989,11 +15381,11 @@
         <v>5.5</v>
       </c>
       <c r="H54" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="Q54" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -15008,7 +15400,7 @@
       </c>
       <c r="X54" t="inlineStr"/>
       <c r="Z54" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
@@ -15035,6 +15427,7 @@
       <c r="AL54" t="inlineStr"/>
       <c r="AM54" t="inlineStr"/>
       <c r="AN54" t="inlineStr"/>
+      <c r="AO54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15065,7 +15458,7 @@
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="Q55" t="n">
-        <v>7.1</v>
+        <v>2.4</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -15080,7 +15473,7 @@
       </c>
       <c r="X55" t="inlineStr"/>
       <c r="Z55" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AA55" t="inlineStr">
         <is>
@@ -15107,6 +15500,7 @@
       <c r="AL55" t="inlineStr"/>
       <c r="AM55" t="inlineStr"/>
       <c r="AN55" t="inlineStr"/>
+      <c r="AO55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15126,22 +15520,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>default-58d2b845</t>
+          <t>default-bc4774ae</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="H56" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="N56" t="inlineStr"/>
       <c r="Q56" t="n">
-        <v>0.9</v>
+        <v>7.9</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Cascade</t>
+          <t>Centennial</t>
         </is>
       </c>
       <c r="U56" t="inlineStr"/>
@@ -15151,8 +15545,11 @@
         </is>
       </c>
       <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="n">
+        <v>76</v>
+      </c>
       <c r="Z56" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
@@ -15161,12 +15558,12 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Bittering</t>
         </is>
       </c>
       <c r="AC56" t="inlineStr">
         <is>
-          <t>Boil</t>
+          <t>Aroma</t>
         </is>
       </c>
       <c r="AD56" t="inlineStr"/>
@@ -15177,8 +15574,8 @@
       <c r="AJ56" t="inlineStr"/>
       <c r="AK56" t="inlineStr"/>
       <c r="AL56" t="inlineStr"/>
-      <c r="AM56" t="inlineStr"/>
       <c r="AN56" t="inlineStr"/>
+      <c r="AO56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -15253,16 +15650,17 @@
       <c r="AK57" t="inlineStr"/>
       <c r="AL57" t="inlineStr"/>
       <c r="AN57" t="inlineStr"/>
+      <c r="AO57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>yiPSN3Y6mmATMzlZ26e4uWlmbGRxaD</t>
+          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>First lager</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -15272,36 +15670,33 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>default-bc4774ae</t>
+          <t>default-b73163ee</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H58" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N58" t="inlineStr"/>
       <c r="Q58" t="n">
-        <v>3.2</v>
+        <v>19.2</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Centennial</t>
+          <t>Hallertauer Mittelfrueh</t>
         </is>
       </c>
       <c r="U58" t="inlineStr"/>
       <c r="W58" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="X58" t="inlineStr"/>
-      <c r="Y58" t="n">
-        <v>76</v>
-      </c>
       <c r="Z58" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="AA58" t="inlineStr">
         <is>
@@ -15310,12 +15705,12 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>Bittering</t>
+          <t>Aroma</t>
         </is>
       </c>
       <c r="AC58" t="inlineStr">
         <is>
-          <t>Aroma</t>
+          <t>Boil</t>
         </is>
       </c>
       <c r="AD58" t="inlineStr"/>
@@ -15326,7 +15721,9 @@
       <c r="AJ58" t="inlineStr"/>
       <c r="AK58" t="inlineStr"/>
       <c r="AL58" t="inlineStr"/>
+      <c r="AM58" t="inlineStr"/>
       <c r="AN58" t="inlineStr"/>
+      <c r="AO58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -15353,11 +15750,11 @@
         <v>4</v>
       </c>
       <c r="H59" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="N59" t="inlineStr"/>
       <c r="Q59" t="n">
-        <v>19.2</v>
+        <v>2.3</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -15372,7 +15769,7 @@
       </c>
       <c r="X59" t="inlineStr"/>
       <c r="Z59" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
@@ -15399,16 +15796,17 @@
       <c r="AL59" t="inlineStr"/>
       <c r="AM59" t="inlineStr"/>
       <c r="AN59" t="inlineStr"/>
+      <c r="AO59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>First lager</t>
+          <t>Smash - Citra</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -15418,44 +15816,51 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>default-b73163ee</t>
+          <t>new-51wCf6O7CNR123kNt0aqW8Oah49aNp</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H60" t="n">
-        <v>10</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
       <c r="Q60" t="n">
-        <v>2.3</v>
-      </c>
+        <v>14.7</v>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr">
         <is>
-          <t>Hallertauer Mittelfrueh</t>
+          <t>Citra</t>
         </is>
       </c>
       <c r="U60" t="inlineStr"/>
+      <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>U.S.</t>
         </is>
       </c>
       <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
       <c r="Z60" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="AA60" t="inlineStr">
         <is>
           <t>Pellet</t>
         </is>
       </c>
-      <c r="AB60" t="inlineStr">
-        <is>
-          <t>Aroma</t>
-        </is>
-      </c>
+      <c r="AB60" t="inlineStr"/>
       <c r="AC60" t="inlineStr">
         <is>
           <t>Boil</t>
@@ -15463,6 +15868,7 @@
       </c>
       <c r="AD60" t="inlineStr"/>
       <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr"/>
       <c r="AG60" t="inlineStr"/>
       <c r="AH60" t="inlineStr"/>
       <c r="AI60" t="inlineStr"/>
@@ -15471,9 +15877,343 @@
       <c r="AL60" t="inlineStr"/>
       <c r="AM60" t="inlineStr"/>
       <c r="AN60" t="inlineStr"/>
+      <c r="AO60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>new-51wCf6O7CNR123kNt0aqW8Oah49aNp</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>12</v>
+      </c>
+      <c r="H61" t="n">
+        <v>60</v>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Citra</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
+      <c r="AJ61" t="inlineStr"/>
+      <c r="AK61" t="inlineStr"/>
+      <c r="AL61" t="inlineStr"/>
+      <c r="AM61" t="inlineStr"/>
+      <c r="AN61" t="inlineStr"/>
+      <c r="AO61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>new-51wCf6O7CNR123kNt0aqW8Oah49aNp</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>12</v>
+      </c>
+      <c r="H62" t="n">
+        <v>80</v>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Citra</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="inlineStr"/>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
+      <c r="AJ62" t="inlineStr"/>
+      <c r="AK62" t="inlineStr"/>
+      <c r="AL62" t="inlineStr"/>
+      <c r="AM62" t="inlineStr"/>
+      <c r="AN62" t="inlineStr"/>
+      <c r="AO62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>new-51wCf6O7CNR123kNt0aqW8Oah49aNp</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>12</v>
+      </c>
+      <c r="H63" t="n">
+        <v>60</v>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Citra</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr"/>
+      <c r="Z63" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="inlineStr"/>
+      <c r="AG63" t="inlineStr"/>
+      <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
+      <c r="AJ63" t="inlineStr"/>
+      <c r="AK63" t="inlineStr"/>
+      <c r="AL63" t="inlineStr"/>
+      <c r="AM63" t="inlineStr"/>
+      <c r="AN63" t="inlineStr"/>
+      <c r="AO63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>new-51wCf6O7CNR123kNt0aqW8Oah49aNp</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>1764889200000</v>
+      </c>
+      <c r="G64" t="n">
+        <v>12</v>
+      </c>
+      <c r="H64" t="n">
+        <v>60</v>
+      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Citra</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr"/>
+      <c r="Z64" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>Dry Hop</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr"/>
+      <c r="AF64" t="inlineStr"/>
+      <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
+      <c r="AJ64" t="inlineStr"/>
+      <c r="AK64" t="inlineStr"/>
+      <c r="AL64" t="inlineStr"/>
+      <c r="AM64" t="inlineStr"/>
+      <c r="AN64" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO64" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN60"/>
+  <autoFilter ref="A1:AO64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15484,7 +16224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL20"/>
+  <dimension ref="A1:AL21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -17749,8 +18489,103 @@
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>default-016efc</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>81</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>American ale yeast producing well balanced beers with low diacetyl and a very clean, crisp end palate. Forms a firm foam head and presents a very good ability to stay in suspension during fermentation.</t>
+        </is>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Fermentis</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="n">
+        <v>28</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="n">
+        <v>16</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Safale American</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>pkg</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL20"/>
+  <autoFilter ref="A1:AL21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17761,7 +18596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB106"/>
+  <dimension ref="A1:AB119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -25905,26 +26740,26 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>default-3b1827</t>
+          <t>default-2302b0</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
+          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
+          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
         </is>
       </c>
       <c r="I96" t="n">
-        <v>1781339598782</v>
+        <v>1781339599069</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -25932,17 +26767,18 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>2</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="b">
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>44</v>
+        <v>94.5</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>Calcium Chloride (CaCl2)</t>
+          <t>Baking Soda (NaHCO3)</t>
         </is>
       </c>
       <c r="Q96" t="b">
@@ -25989,26 +26825,26 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>default-1f88df</t>
+          <t>default-3b1827</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
+          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
+          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>1781339597373</v>
+        <v>1781339598782</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -26016,18 +26852,17 @@
         </is>
       </c>
       <c r="K97" t="n">
-        <v>2</v>
-      </c>
-      <c r="L97" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
       <c r="M97" t="b">
         <v>0</v>
       </c>
       <c r="N97" t="n">
-        <v>941.2</v>
+        <v>44</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Gypsum (CaSO4)</t>
+          <t>Calcium Chloride (CaCl2)</t>
         </is>
       </c>
       <c r="Q97" t="b">
@@ -26074,26 +26909,26 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>default-1f88df</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
+          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
+          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>1781339599470</v>
+        <v>1781339597373</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -26101,20 +26936,18 @@
         </is>
       </c>
       <c r="K98" t="n">
-        <v>2</v>
-      </c>
-      <c r="L98" t="n">
-        <v>80</v>
-      </c>
+        <v>4.6</v>
+      </c>
+      <c r="L98" t="inlineStr"/>
       <c r="M98" t="b">
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>342.5</v>
+        <v>941.2</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
+          <t>Gypsum (CaSO4)</t>
         </is>
       </c>
       <c r="Q98" t="b">
@@ -26127,7 +26960,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
@@ -26161,69 +26994,70 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>default-5adf6e</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>z82GocB6JPQV699Mhx10blYxb69kZE</t>
+          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>1775809151504</v>
+        <v>1781339599470</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>3.0.0</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="K99" t="n">
-        <v>5</v>
-      </c>
-      <c r="L99" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="L99" t="n">
+        <v>80</v>
+      </c>
       <c r="M99" t="b">
         <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>5</v>
+        <v>342.5</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Irish Moss</t>
-        </is>
-      </c>
-      <c r="P99" t="n">
-        <v>10</v>
+          <t>Lactic Acid</t>
+        </is>
       </c>
       <c r="Q99" t="b">
         <v>0</v>
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Water Agent</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>Boil</t>
-        </is>
-      </c>
-      <c r="U99" t="inlineStr"/>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U99" t="b">
+        <v>1</v>
+      </c>
       <c r="Y99" t="inlineStr"/>
       <c r="Z99" t="inlineStr"/>
       <c r="AA99" t="inlineStr"/>
@@ -26247,26 +27081,26 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>default-yn-wln1000</t>
+          <t>default-5adf6e</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>naf4Kaq8Bj5vVUHIgICtzv9zYVFplp</t>
+          <t>z82GocB6JPQV699Mhx10blYxb69kZE</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>1775809134067</v>
+        <v>1775809151504</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -26274,18 +27108,18 @@
         </is>
       </c>
       <c r="K100" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="b">
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Yeast Nutrient (WLN1000)</t>
+          <t>Irish Moss</t>
         </is>
       </c>
       <c r="P100" t="n">
@@ -26296,7 +27130,7 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
@@ -26310,15 +27144,7 @@
         </is>
       </c>
       <c r="U100" t="inlineStr"/>
-      <c r="V100" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="Y100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">White Labs Yeast Nutrient is used to increase the health of yeast, this improves fermentation and re-pitching performance. It contains diammonium phosphate (DAP), essential vitamins and co-factors, nitrogen, amino acids, proteins, peptides, and minerals. An effective boost for first and/or late-generation yeast slurry. If the grist is not 100% malt, then White Labs Yeast Nutrient can help make up for the lack of nutrients.
-We recommend using traditional finings agents for most fermentations. If you are still struggling with unwanted haze, filtration may be necessary. </t>
-        </is>
-      </c>
+      <c r="Y100" t="inlineStr"/>
       <c r="Z100" t="inlineStr"/>
       <c r="AA100" t="inlineStr"/>
       <c r="AB100" t="inlineStr"/>
@@ -26326,12 +27152,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+          <t>yiPSN3Y6mmATMzlZ26e4uWlmbGRxaD</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>First lager</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -26341,53 +27167,56 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 191000000, "_seconds": 1706434206}</t>
+          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>default-bk9j78</t>
+          <t>default-yn-wln1000</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>1PMknHJZdv0oQ7VqqIQ2rbYXMm9N5D</t>
+          <t>naf4Kaq8Bj5vVUHIgICtzv9zYVFplp</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 260000000, "_seconds": 1712314610}</t>
+          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>1712314610260</v>
+        <v>1775809134067</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>2.10.6</t>
+          <t>3.0.0</t>
         </is>
       </c>
       <c r="K101" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="b">
         <v>0</v>
       </c>
       <c r="N101" t="n">
-        <v>-5</v>
+        <v>80</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Canning Salt (NaCl)</t>
-        </is>
+          <t>Yeast Nutrient (WLN1000)</t>
+        </is>
+      </c>
+      <c r="P101" t="n">
+        <v>10</v>
       </c>
       <c r="Q101" t="b">
         <v>0</v>
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>Water Agent</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
@@ -26397,16 +27226,19 @@
       </c>
       <c r="T101" t="inlineStr">
         <is>
-          <t>Mash</t>
-        </is>
-      </c>
-      <c r="U101" t="b">
-        <v>1</v>
-      </c>
-      <c r="V101" t="inlineStr"/>
-      <c r="W101" t="inlineStr"/>
-      <c r="X101" t="inlineStr"/>
-      <c r="Y101" t="inlineStr"/>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr"/>
+      <c r="V101" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">White Labs Yeast Nutrient is used to increase the health of yeast, this improves fermentation and re-pitching performance. It contains diammonium phosphate (DAP), essential vitamins and co-factors, nitrogen, amino acids, proteins, peptides, and minerals. An effective boost for first and/or late-generation yeast slurry. If the grist is not 100% malt, then White Labs Yeast Nutrient can help make up for the lack of nutrients.
+We recommend using traditional finings agents for most fermentations. If you are still struggling with unwanted haze, filtration may be necessary. </t>
+        </is>
+      </c>
       <c r="Z101" t="inlineStr"/>
       <c r="AA101" t="inlineStr"/>
       <c r="AB101" t="inlineStr"/>
@@ -26429,26 +27261,26 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+          <t>{"_nanoseconds": 191000000, "_seconds": 1706434206}</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>default-1f88df</t>
+          <t>default-bk9j78</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>lwPgFpUrns6MH8XqOw1PIDi3cAnGBV</t>
+          <t>1PMknHJZdv0oQ7VqqIQ2rbYXMm9N5D</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 450000000, "_seconds": 1712314609}</t>
+          <t>{"_nanoseconds": 260000000, "_seconds": 1712314610}</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>1712314609450</v>
+        <v>1712314610260</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -26456,18 +27288,18 @@
         </is>
       </c>
       <c r="K102" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="b">
         <v>0</v>
       </c>
       <c r="N102" t="n">
-        <v>-12</v>
+        <v>-5</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Gypsum (CaSO4)</t>
+          <t>Canning Salt (NaCl)</t>
         </is>
       </c>
       <c r="Q102" t="b">
@@ -26491,6 +27323,9 @@
       <c r="U102" t="b">
         <v>1</v>
       </c>
+      <c r="V102" t="inlineStr"/>
+      <c r="W102" t="inlineStr"/>
+      <c r="X102" t="inlineStr"/>
       <c r="Y102" t="inlineStr"/>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr"/>
@@ -26514,47 +27349,45 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>default-1f88df</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Wtg8GXKfWxQjJGGYxmK7mUYTRcgSh9</t>
+          <t>lwPgFpUrns6MH8XqOw1PIDi3cAnGBV</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 450000000, "_seconds": 1712314609}</t>
         </is>
       </c>
       <c r="I103" t="n">
-        <v>1706434207828</v>
+        <v>1712314609450</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>2.10.5</t>
+          <t>2.10.6</t>
         </is>
       </c>
       <c r="K103" t="n">
-        <v>3</v>
-      </c>
-      <c r="L103" t="n">
-        <v>80</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="L103" t="inlineStr"/>
       <c r="M103" t="b">
         <v>0</v>
       </c>
       <c r="N103" t="n">
-        <v>-4</v>
+        <v>-12</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
+          <t>Gypsum (CaSO4)</t>
         </is>
       </c>
       <c r="Q103" t="b">
@@ -26567,7 +27400,7 @@
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -26578,9 +27411,6 @@
       <c r="U103" t="b">
         <v>1</v>
       </c>
-      <c r="V103" t="inlineStr"/>
-      <c r="W103" t="inlineStr"/>
-      <c r="X103" t="inlineStr"/>
       <c r="Y103" t="inlineStr"/>
       <c r="Z103" t="inlineStr"/>
       <c r="AA103" t="inlineStr"/>
@@ -26602,49 +27432,75 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>default-6bc446</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Wtg8GXKfWxQjJGGYxmK7mUYTRcgSh9</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>1706434207828</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2.10.5</t>
+        </is>
+      </c>
       <c r="K104" t="n">
-        <v>5</v>
-      </c>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L104" t="n">
+        <v>80</v>
+      </c>
+      <c r="M104" t="b">
+        <v>0</v>
+      </c>
+      <c r="N104" t="n">
+        <v>-4</v>
+      </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Biofine Clear</t>
-        </is>
-      </c>
-      <c r="P104" t="n">
-        <v>15</v>
+          <t>Lactic Acid</t>
+        </is>
       </c>
       <c r="Q104" t="b">
+        <v>0</v>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U104" t="b">
         <v>1</v>
       </c>
-      <c r="R104" t="inlineStr">
-        <is>
-          <t>Fining</t>
-        </is>
-      </c>
-      <c r="S104" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
-      <c r="T104" t="inlineStr">
-        <is>
-          <t>Boil</t>
-        </is>
-      </c>
-      <c r="U104" t="inlineStr"/>
+      <c r="V104" t="inlineStr"/>
+      <c r="W104" t="inlineStr"/>
+      <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr"/>
       <c r="Z104" t="inlineStr"/>
       <c r="AA104" t="inlineStr"/>
@@ -26666,63 +27522,41 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>default-yn1j28sf</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>n9o5cFAQDFJBRKVV6LFjrQgK6Vnlsr</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 742000000, "_seconds": 1712314613}</t>
-        </is>
-      </c>
-      <c r="I105" t="n">
-        <v>1712314613742</v>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>2.10.6</t>
-        </is>
-      </c>
+          <t>default-6bc446</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
       <c r="K105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L105" t="inlineStr"/>
-      <c r="M105" t="b">
-        <v>0</v>
-      </c>
-      <c r="N105" t="n">
-        <v>-11</v>
-      </c>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr">
         <is>
-          <t>Yeast Nutrients</t>
+          <t>Biofine Clear</t>
         </is>
       </c>
       <c r="P105" t="n">
         <v>15</v>
       </c>
       <c r="Q105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -26754,63 +27588,66 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 538000000, "_seconds": 1697269076}</t>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>default-90c63c</t>
+          <t>default-yn1j28sf</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>n39qcIsSvY0mhj8mb0KhJHE9df0bXd</t>
+          <t>n9o5cFAQDFJBRKVV6LFjrQgK6Vnlsr</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 300000000, "_seconds": 1704369578}</t>
+          <t>{"_nanoseconds": 742000000, "_seconds": 1712314613}</t>
         </is>
       </c>
       <c r="I106" t="n">
-        <v>1704369578300</v>
+        <v>1712314613742</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>2.10.4</t>
+          <t>2.10.6</t>
         </is>
       </c>
       <c r="K106" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="b">
         <v>0</v>
       </c>
       <c r="N106" t="n">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Gelatin</t>
-        </is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P106" t="n">
+        <v>15</v>
       </c>
       <c r="Q106" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Boil</t>
         </is>
       </c>
       <c r="U106" t="inlineStr"/>
@@ -26819,8 +27656,865 @@
       <c r="AA106" t="inlineStr"/>
       <c r="AB106" t="inlineStr"/>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>First lager</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 538000000, "_seconds": 1697269076}</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>default-90c63c</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>n39qcIsSvY0mhj8mb0KhJHE9df0bXd</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 300000000, "_seconds": 1704369578}</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>1704369578300</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>2.10.4</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>5</v>
+      </c>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="b">
+        <v>0</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Gelatin</t>
+        </is>
+      </c>
+      <c r="Q107" t="b">
+        <v>1</v>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr"/>
+      <c r="Y107" t="inlineStr"/>
+      <c r="Z107" t="inlineStr"/>
+      <c r="AA107" t="inlineStr"/>
+      <c r="AB107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Calcium Chloride</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr"/>
+      <c r="V108" t="inlineStr"/>
+      <c r="W108" t="inlineStr"/>
+      <c r="X108" t="inlineStr"/>
+      <c r="Y108" t="inlineStr"/>
+      <c r="Z108" t="inlineStr"/>
+      <c r="AA108" t="inlineStr"/>
+      <c r="AB108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="n">
+        <v>10</v>
+      </c>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Epsom Salt (MgSO4)</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr"/>
+      <c r="V109" t="inlineStr"/>
+      <c r="W109" t="inlineStr"/>
+      <c r="X109" t="inlineStr"/>
+      <c r="Y109" t="inlineStr"/>
+      <c r="Z109" t="inlineStr"/>
+      <c r="AA109" t="inlineStr"/>
+      <c r="AB109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Gypsum (Calcium Sulfate)</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr"/>
+      <c r="V110" t="inlineStr"/>
+      <c r="W110" t="inlineStr"/>
+      <c r="X110" t="inlineStr"/>
+      <c r="Y110" t="inlineStr"/>
+      <c r="Z110" t="inlineStr"/>
+      <c r="AA110" t="inlineStr"/>
+      <c r="AB110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="L111" t="n">
+        <v>80</v>
+      </c>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q111" t="b">
+        <v>0</v>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U111" t="b">
+        <v>1</v>
+      </c>
+      <c r="V111" t="inlineStr"/>
+      <c r="W111" t="inlineStr"/>
+      <c r="X111" t="inlineStr"/>
+      <c r="Y111" t="inlineStr"/>
+      <c r="Z111" t="inlineStr"/>
+      <c r="AA111" t="inlineStr"/>
+      <c r="AB111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr"/>
+      <c r="V112" t="inlineStr"/>
+      <c r="W112" t="inlineStr"/>
+      <c r="X112" t="inlineStr"/>
+      <c r="Y112" t="inlineStr"/>
+      <c r="Z112" t="inlineStr"/>
+      <c r="AA112" t="inlineStr"/>
+      <c r="AB112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="L113" t="n">
+        <v>80</v>
+      </c>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q113" t="b">
+        <v>0</v>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Sparge</t>
+        </is>
+      </c>
+      <c r="U113" t="b">
+        <v>1</v>
+      </c>
+      <c r="V113" t="inlineStr"/>
+      <c r="W113" t="inlineStr"/>
+      <c r="X113" t="inlineStr"/>
+      <c r="Y113" t="inlineStr"/>
+      <c r="Z113" t="inlineStr"/>
+      <c r="AA113" t="inlineStr"/>
+      <c r="AB113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Calcium Chloride</t>
+        </is>
+      </c>
+      <c r="P114" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr"/>
+      <c r="V114" t="inlineStr"/>
+      <c r="W114" t="inlineStr"/>
+      <c r="X114" t="inlineStr"/>
+      <c r="Y114" t="inlineStr"/>
+      <c r="Z114" t="inlineStr"/>
+      <c r="AA114" t="inlineStr"/>
+      <c r="AB114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Epsom Salt (MgSO4)</t>
+        </is>
+      </c>
+      <c r="P115" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q115" t="inlineStr"/>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr"/>
+      <c r="V115" t="inlineStr"/>
+      <c r="W115" t="inlineStr"/>
+      <c r="X115" t="inlineStr"/>
+      <c r="Y115" t="inlineStr"/>
+      <c r="Z115" t="inlineStr"/>
+      <c r="AA115" t="inlineStr"/>
+      <c r="AB115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Gypsum (Calcium Sulfate)</t>
+        </is>
+      </c>
+      <c r="P116" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr"/>
+      <c r="V116" t="inlineStr"/>
+      <c r="W116" t="inlineStr"/>
+      <c r="X116" t="inlineStr"/>
+      <c r="Y116" t="inlineStr"/>
+      <c r="Z116" t="inlineStr"/>
+      <c r="AA116" t="inlineStr"/>
+      <c r="AB116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="P117" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr"/>
+      <c r="V117" t="inlineStr"/>
+      <c r="W117" t="inlineStr"/>
+      <c r="X117" t="inlineStr"/>
+      <c r="Y117" t="inlineStr"/>
+      <c r="Z117" t="inlineStr"/>
+      <c r="AA117" t="inlineStr"/>
+      <c r="AB117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>new-TUfxqCta0ITj3uHT8vfAbVIfLtzqyA</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="n">
+        <v>2</v>
+      </c>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Protafloc</t>
+        </is>
+      </c>
+      <c r="P118" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>tbsp</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U118" t="inlineStr"/>
+      <c r="V118" t="inlineStr"/>
+      <c r="W118" t="inlineStr"/>
+      <c r="X118" t="inlineStr"/>
+      <c r="Y118" t="inlineStr"/>
+      <c r="Z118" t="inlineStr"/>
+      <c r="AA118" t="inlineStr"/>
+      <c r="AB118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Smash - Citra</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>new-Xe5CxkyeaTwnbVay8pIU6ai8XycVKB</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="n">
+        <v>2</v>
+      </c>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Yeast Nutrient</t>
+        </is>
+      </c>
+      <c r="P119" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>tsp</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr"/>
+      <c r="V119" t="inlineStr"/>
+      <c r="W119" t="inlineStr"/>
+      <c r="X119" t="inlineStr"/>
+      <c r="Y119" t="inlineStr"/>
+      <c r="Z119" t="inlineStr"/>
+      <c r="AA119" t="inlineStr"/>
+      <c r="AB119" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB106"/>
+  <autoFilter ref="A1:AB119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-07-16 04:58 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$76</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AO$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AO$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1833,8 +1833,75 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ernst Gouws</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1.04757289</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>First attempt at saison. 
+Using farmhouse yeast. 
+Start at 24 and freerise / slow rise to 28 hopefully to get more flavor from the yeast. 
+Table sugar to get it dryer.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P21"/>
+  <autoFilter ref="A1:P22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1845,7 +1912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT76"/>
+  <dimension ref="A1:AT79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10021,8 +10088,304 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>default-c3ff8bb88f9</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>tqtVycoLMiKmJMplyu7GCIAsAeeETL</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 476000000, "_seconds": 1781339591}</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>1781339591476</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Base (Pilsner)</t>
+        </is>
+      </c>
+      <c r="X77" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>Swaen Pilsner</t>
+        </is>
+      </c>
+      <c r="AE77" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF77" t="inlineStr"/>
+      <c r="AG77" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH77" t="n">
+        <v>81.97</v>
+      </c>
+      <c r="AI77" t="n">
+        <v>1.0368</v>
+      </c>
+      <c r="AJ77" t="n">
+        <v>80</v>
+      </c>
+      <c r="AL77" t="inlineStr"/>
+      <c r="AM77" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN77" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO77" t="inlineStr"/>
+      <c r="AP77" t="inlineStr"/>
+      <c r="AQ77" t="inlineStr"/>
+      <c r="AR77" t="inlineStr"/>
+      <c r="AS77" t="inlineStr"/>
+      <c r="AT77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>default-d9e04639a2c</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>zNojkfDZoro1z7t7fMQtUDJKvZGT6s</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 852000000, "_seconds": 1781339591}</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>1781339591852</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>Base (Vienna)</t>
+        </is>
+      </c>
+      <c r="X78" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>Swaen Vienna</t>
+        </is>
+      </c>
+      <c r="AE78" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF78" t="inlineStr"/>
+      <c r="AG78" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH78" t="n">
+        <v>11.48</v>
+      </c>
+      <c r="AI78" t="n">
+        <v>1.03588</v>
+      </c>
+      <c r="AJ78" t="n">
+        <v>78</v>
+      </c>
+      <c r="AL78" t="inlineStr"/>
+      <c r="AM78" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN78" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO78" t="inlineStr"/>
+      <c r="AP78" t="inlineStr"/>
+      <c r="AQ78" t="inlineStr"/>
+      <c r="AR78" t="inlineStr"/>
+      <c r="AS78" t="inlineStr"/>
+      <c r="AT78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 526000000, "_seconds": 1719746358}</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>default-132c22b</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>feD3na0a4sxySPUBRKwyBrSewo4G5I</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 383000000, "_seconds": 1772634460}</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>1772634460383</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>2.20.2</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M79" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>1</v>
+      </c>
+      <c r="X79" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>Sugar, Table (Sucrose)</t>
+        </is>
+      </c>
+      <c r="AE79" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF79" t="inlineStr"/>
+      <c r="AG79" t="inlineStr"/>
+      <c r="AH79" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="AI79" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="AJ79" t="n">
+        <v>100</v>
+      </c>
+      <c r="AL79" t="inlineStr"/>
+      <c r="AM79" t="inlineStr"/>
+      <c r="AN79" t="inlineStr">
+        <is>
+          <t>Sugar</t>
+        </is>
+      </c>
+      <c r="AO79" t="inlineStr"/>
+      <c r="AP79" t="inlineStr"/>
+      <c r="AQ79" t="inlineStr"/>
+      <c r="AR79" t="inlineStr"/>
+      <c r="AS79" t="inlineStr"/>
+      <c r="AT79" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT76"/>
+  <autoFilter ref="A1:AT79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10033,7 +10396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO64"/>
+  <dimension ref="A1:AO67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16212,8 +16575,350 @@
         <v>1</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>default-NrD3kYzu8ONSucGjXgHxRcgSUwk2aK</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H65" t="n">
+        <v>20</v>
+      </c>
+      <c r="J65" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="K65" t="n">
+        <v>11</v>
+      </c>
+      <c r="L65" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M65" t="n">
+        <v>17</v>
+      </c>
+      <c r="N65" t="b">
+        <v>0</v>
+      </c>
+      <c r="P65" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="S65" t="n">
+        <v>33</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Saaz</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Saaz is the famous aroma landrace variety originating in the Czech area of the same name. It has very mild, pleasant noble hoppy notes perfectly suited for and defines the Czech-style pilsner beers.
+Pedigree Czech landrace variety Aroma Classic noble aroma hop with long and strong tradition associated with classic pilsner beer.</t>
+        </is>
+      </c>
+      <c r="V65" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr"/>
+      <c r="Z65" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr"/>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 967000000, "_seconds": 1775807186}</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>wgmsfM7hAArpDzCYHBWiW6iwLQheal</t>
+        </is>
+      </c>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 703000000, "_seconds": 1781070146}</t>
+        </is>
+      </c>
+      <c r="AJ65" t="n">
+        <v>1781070146703</v>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL65" t="n">
+        <v>150</v>
+      </c>
+      <c r="AM65" t="inlineStr"/>
+      <c r="AN65" t="inlineStr"/>
+      <c r="AO65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>default-J80zzFn0TQEAwwaQuzMQsRYzrIvBOC</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H66" t="n">
+        <v>10</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N66" t="b">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Hallertau Perle</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>A dual-purpose hop that offers great bittering properties as well as a well-rounded aroma profile. Aroma: Herbal - tea, pepper, floral, citrus, earthy, woody, grassy, caramel Alpha Acid: 4.0 - 9.0% Beta Acid: 2.5 - 4.5% Total Oil: 0.5 - 1.3 ml/100g</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr"/>
+      <c r="Z66" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr"/>
+      <c r="AF66" t="n">
+        <v>2024</v>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 223000000, "_seconds": 1778682625}</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
+          <t>7XQ2gOtWELwAzHhtmwIarzOqsdzdzE</t>
+        </is>
+      </c>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 684000000, "_seconds": 1781339595}</t>
+        </is>
+      </c>
+      <c r="AJ66" t="n">
+        <v>1781339595684</v>
+      </c>
+      <c r="AK66" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL66" t="n">
+        <v>170</v>
+      </c>
+      <c r="AM66" t="inlineStr"/>
+      <c r="AN66" t="inlineStr"/>
+      <c r="AO66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>default-NrD3kYzu8ONSucGjXgHxRcgSUwk2aK</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>20</v>
+      </c>
+      <c r="J67" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="K67" t="n">
+        <v>11</v>
+      </c>
+      <c r="L67" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M67" t="n">
+        <v>17</v>
+      </c>
+      <c r="N67" t="b">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S67" t="n">
+        <v>33</v>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Saaz</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Saaz is the famous aroma landrace variety originating in the Czech area of the same name. It has very mild, pleasant noble hoppy notes perfectly suited for and defines the Czech-style pilsner beers.
+Pedigree Czech landrace variety Aroma Classic noble aroma hop with long and strong tradition associated with classic pilsner beer.</t>
+        </is>
+      </c>
+      <c r="V67" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr"/>
+      <c r="Z67" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr"/>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 967000000, "_seconds": 1775807186}</t>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
+          <t>wgmsfM7hAArpDzCYHBWiW6iwLQheal</t>
+        </is>
+      </c>
+      <c r="AI67" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 703000000, "_seconds": 1781070146}</t>
+        </is>
+      </c>
+      <c r="AJ67" t="n">
+        <v>1781070146703</v>
+      </c>
+      <c r="AK67" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL67" t="n">
+        <v>150</v>
+      </c>
+      <c r="AM67" t="inlineStr"/>
+      <c r="AN67" t="inlineStr"/>
+      <c r="AO67" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AO64"/>
+  <autoFilter ref="A1:AO67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16224,7 +16929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL21"/>
+  <dimension ref="A1:AL22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18584,8 +19289,133 @@
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>default-8FqpUdhfVGoKyF5z0R03cRiQBTlTqo</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>default-lallemand-koln</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>80</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Vigorous fermentation that can be completed in 5 days</t>
+        </is>
+      </c>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Lallemand (LalBrew)</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>13</v>
+      </c>
+      <c r="S22" t="n">
+        <v>30</v>
+      </c>
+      <c r="U22" t="n">
+        <v>20</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Farmhouse</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>pkg</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>kölsch-style, neutral ales</t>
+        </is>
+      </c>
+      <c r="AF22" t="n">
+        <v>60</v>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 856000000, "_seconds": 1784057989}</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>ExrXBelZBDAWJ8Bul57dLy2OgQdtkF</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 856000000, "_seconds": 1784057989}</t>
+        </is>
+      </c>
+      <c r="AJ22" t="n">
+        <v>1784057989856</v>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL22" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL21"/>
+  <autoFilter ref="A1:AL22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18596,7 +19426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB119"/>
+  <dimension ref="A1:AB126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -28513,8 +29343,609 @@
       <c r="AA119" t="inlineStr"/>
       <c r="AB119" t="inlineStr"/>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>default-2302b0</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>1781339599069</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="b">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Baking Soda (NaHCO3)</t>
+        </is>
+      </c>
+      <c r="Q120" t="b">
+        <v>0</v>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U120" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y120" t="inlineStr"/>
+      <c r="Z120" t="inlineStr"/>
+      <c r="AA120" t="inlineStr"/>
+      <c r="AB120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>default-3b1827</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>1781339598782</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>2</v>
+      </c>
+      <c r="M121" t="b">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>44</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Calcium Chloride (CaCl2)</t>
+        </is>
+      </c>
+      <c r="Q121" t="b">
+        <v>0</v>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U121" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y121" t="inlineStr"/>
+      <c r="Z121" t="inlineStr"/>
+      <c r="AA121" t="inlineStr"/>
+      <c r="AB121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 459000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>default-4e9d62</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>baUPFv7WEZjl8hB5Cj0fMBSpkrFQ3R</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 229000000, "_seconds": 1704369577}</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>1704369577229</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2.10.4</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>2</v>
+      </c>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="b">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Epsom Salt (MgSO4)</t>
+        </is>
+      </c>
+      <c r="Q122" t="b">
+        <v>0</v>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U122" t="b">
+        <v>1</v>
+      </c>
+      <c r="V122" t="inlineStr"/>
+      <c r="W122" t="inlineStr"/>
+      <c r="X122" t="inlineStr"/>
+      <c r="Y122" t="inlineStr"/>
+      <c r="Z122" t="inlineStr"/>
+      <c r="AA122" t="inlineStr"/>
+      <c r="AB122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>default-1f88df</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>1781339597373</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>3</v>
+      </c>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="b">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
+        <v>941.2</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Gypsum (CaSO4)</t>
+        </is>
+      </c>
+      <c r="Q123" t="b">
+        <v>0</v>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U123" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y123" t="inlineStr"/>
+      <c r="Z123" t="inlineStr"/>
+      <c r="AA123" t="inlineStr"/>
+      <c r="AB123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>1781339599470</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L124" t="n">
+        <v>80</v>
+      </c>
+      <c r="M124" t="b">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>342.5</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q124" t="b">
+        <v>0</v>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U124" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y124" t="inlineStr"/>
+      <c r="Z124" t="inlineStr"/>
+      <c r="AA124" t="inlineStr"/>
+      <c r="AB124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>default-yn1j28sf</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>92ChBNr2k0grfMSG7XIrynIVfyh02o</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 221000000, "_seconds": 1781339600}</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>1781339600221</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>5</v>
+      </c>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="b">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>33</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P125" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q125" t="b">
+        <v>0</v>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U125" t="inlineStr"/>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr"/>
+      <c r="AB125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>default-5adf6e</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>ntpZTYp6GFzhrk8IfC1bCJaKbHeIyI</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 65000000, "_seconds": 1778997170}</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>1778997170065</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>5</v>
+      </c>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="b">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Irish Moss</t>
+        </is>
+      </c>
+      <c r="P126" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q126" t="b">
+        <v>0</v>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U126" t="inlineStr"/>
+      <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB119"/>
+  <autoFilter ref="A1:AB126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-07-21 05:18 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -1682,7 +1682,7 @@
         <v>5.38</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>30.1</v>
+        <v>28.8</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>5.7</v>
@@ -15636,7 +15636,7 @@
         <v>6.3</v>
       </c>
       <c r="H53" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J53" t="n">
         <v>3.5</v>
@@ -15648,7 +15648,7 @@
         <v>30</v>
       </c>
       <c r="Q53" t="n">
-        <v>15</v>
+        <v>12.9</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -15817,11 +15817,11 @@
         <v>10</v>
       </c>
       <c r="H55" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="Q55" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update: 2026-07-27 05:47 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AO$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19532,7 +19532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB125"/>
+  <dimension ref="A1:AB124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -27587,26 +27587,26 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>default-2302b0</t>
+          <t>default-3b1827</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
         </is>
       </c>
       <c r="I95" t="n">
-        <v>1781339599069</v>
+        <v>1781339598782</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -27614,18 +27614,17 @@
         </is>
       </c>
       <c r="K95" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L95" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
       <c r="M95" t="b">
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>94.5</v>
+        <v>44</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Baking Soda (NaHCO3)</t>
+          <t>Calcium Chloride (CaCl2)</t>
         </is>
       </c>
       <c r="Q95" t="b">
@@ -27672,26 +27671,26 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>default-3b1827</t>
+          <t>default-1f88df</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
+          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
+          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
         </is>
       </c>
       <c r="I96" t="n">
-        <v>1781339598782</v>
+        <v>1781339597373</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -27699,17 +27698,18 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>3.5</v>
-      </c>
+        <v>4.5</v>
+      </c>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="b">
         <v>0</v>
       </c>
       <c r="N96" t="n">
-        <v>44</v>
+        <v>941.2</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>Calcium Chloride (CaCl2)</t>
+          <t>Gypsum (CaSO4)</t>
         </is>
       </c>
       <c r="Q96" t="b">
@@ -27756,26 +27756,26 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>default-1f88df</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
+          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
+          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>1781339597373</v>
+        <v>1781339599470</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -27783,18 +27783,20 @@
         </is>
       </c>
       <c r="K97" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="L97" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="L97" t="n">
+        <v>80</v>
+      </c>
       <c r="M97" t="b">
         <v>0</v>
       </c>
       <c r="N97" t="n">
-        <v>941.2</v>
+        <v>342.5</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Gypsum (CaSO4)</t>
+          <t>Lactic Acid</t>
         </is>
       </c>
       <c r="Q97" t="b">
@@ -27807,7 +27809,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T97" t="inlineStr">
@@ -27841,70 +27843,69 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>default-5adf6e</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
+          <t>z82GocB6JPQV699Mhx10blYxb69kZE</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>1781339599470</v>
+        <v>1775809151504</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>3.0.1</t>
+          <t>3.0.0</t>
         </is>
       </c>
       <c r="K98" t="n">
-        <v>2</v>
-      </c>
-      <c r="L98" t="n">
-        <v>80</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L98" t="inlineStr"/>
       <c r="M98" t="b">
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>342.5</v>
+        <v>5</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
-        </is>
+          <t>Irish Moss</t>
+        </is>
+      </c>
+      <c r="P98" t="n">
+        <v>10</v>
       </c>
       <c r="Q98" t="b">
         <v>0</v>
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>Water Agent</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>Mash</t>
-        </is>
-      </c>
-      <c r="U98" t="b">
-        <v>1</v>
-      </c>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr"/>
       <c r="Y98" t="inlineStr"/>
       <c r="Z98" t="inlineStr"/>
       <c r="AA98" t="inlineStr"/>
@@ -27928,26 +27929,26 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>default-5adf6e</t>
+          <t>default-yn-wln1000</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>z82GocB6JPQV699Mhx10blYxb69kZE</t>
+          <t>naf4Kaq8Bj5vVUHIgICtzv9zYVFplp</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>1775809151504</v>
+        <v>1775809134067</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -27955,18 +27956,18 @@
         </is>
       </c>
       <c r="K99" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="b">
         <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Irish Moss</t>
+          <t>Yeast Nutrient (WLN1000)</t>
         </is>
       </c>
       <c r="P99" t="n">
@@ -27977,7 +27978,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
@@ -27991,7 +27992,15 @@
         </is>
       </c>
       <c r="U99" t="inlineStr"/>
-      <c r="Y99" t="inlineStr"/>
+      <c r="V99" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">White Labs Yeast Nutrient is used to increase the health of yeast, this improves fermentation and re-pitching performance. It contains diammonium phosphate (DAP), essential vitamins and co-factors, nitrogen, amino acids, proteins, peptides, and minerals. An effective boost for first and/or late-generation yeast slurry. If the grist is not 100% malt, then White Labs Yeast Nutrient can help make up for the lack of nutrients.
+We recommend using traditional finings agents for most fermentations. If you are still struggling with unwanted haze, filtration may be necessary. </t>
+        </is>
+      </c>
       <c r="Z99" t="inlineStr"/>
       <c r="AA99" t="inlineStr"/>
       <c r="AB99" t="inlineStr"/>
@@ -27999,12 +28008,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>yiPSN3Y6mmATMzlZ26e4uWlmbGRxaD</t>
+          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>First lager</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -28014,56 +28023,53 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
+          <t>{"_nanoseconds": 191000000, "_seconds": 1706434206}</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>default-yn-wln1000</t>
+          <t>default-bk9j78</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>naf4Kaq8Bj5vVUHIgICtzv9zYVFplp</t>
+          <t>1PMknHJZdv0oQ7VqqIQ2rbYXMm9N5D</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 67000000, "_seconds": 1775809134}</t>
+          <t>{"_nanoseconds": 260000000, "_seconds": 1712314610}</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>1775809134067</v>
+        <v>1712314610260</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>3.0.0</t>
+          <t>2.10.6</t>
         </is>
       </c>
       <c r="K100" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="b">
         <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>80</v>
+        <v>-5</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Yeast Nutrient (WLN1000)</t>
-        </is>
-      </c>
-      <c r="P100" t="n">
-        <v>10</v>
+          <t>Canning Salt (NaCl)</t>
+        </is>
       </c>
       <c r="Q100" t="b">
         <v>0</v>
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Water Agent</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
@@ -28073,19 +28079,16 @@
       </c>
       <c r="T100" t="inlineStr">
         <is>
-          <t>Boil</t>
-        </is>
-      </c>
-      <c r="U100" t="inlineStr"/>
-      <c r="V100" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="Y100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">White Labs Yeast Nutrient is used to increase the health of yeast, this improves fermentation and re-pitching performance. It contains diammonium phosphate (DAP), essential vitamins and co-factors, nitrogen, amino acids, proteins, peptides, and minerals. An effective boost for first and/or late-generation yeast slurry. If the grist is not 100% malt, then White Labs Yeast Nutrient can help make up for the lack of nutrients.
-We recommend using traditional finings agents for most fermentations. If you are still struggling with unwanted haze, filtration may be necessary. </t>
-        </is>
-      </c>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U100" t="b">
+        <v>1</v>
+      </c>
+      <c r="V100" t="inlineStr"/>
+      <c r="W100" t="inlineStr"/>
+      <c r="X100" t="inlineStr"/>
+      <c r="Y100" t="inlineStr"/>
       <c r="Z100" t="inlineStr"/>
       <c r="AA100" t="inlineStr"/>
       <c r="AB100" t="inlineStr"/>
@@ -28108,26 +28111,26 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 191000000, "_seconds": 1706434206}</t>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>default-bk9j78</t>
+          <t>default-1f88df</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>1PMknHJZdv0oQ7VqqIQ2rbYXMm9N5D</t>
+          <t>lwPgFpUrns6MH8XqOw1PIDi3cAnGBV</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 260000000, "_seconds": 1712314610}</t>
+          <t>{"_nanoseconds": 450000000, "_seconds": 1712314609}</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>1712314610260</v>
+        <v>1712314609450</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -28135,18 +28138,18 @@
         </is>
       </c>
       <c r="K101" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="b">
         <v>0</v>
       </c>
       <c r="N101" t="n">
-        <v>-5</v>
+        <v>-12</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Canning Salt (NaCl)</t>
+          <t>Gypsum (CaSO4)</t>
         </is>
       </c>
       <c r="Q101" t="b">
@@ -28170,9 +28173,6 @@
       <c r="U101" t="b">
         <v>1</v>
       </c>
-      <c r="V101" t="inlineStr"/>
-      <c r="W101" t="inlineStr"/>
-      <c r="X101" t="inlineStr"/>
       <c r="Y101" t="inlineStr"/>
       <c r="Z101" t="inlineStr"/>
       <c r="AA101" t="inlineStr"/>
@@ -28196,45 +28196,47 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>default-1f88df</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>lwPgFpUrns6MH8XqOw1PIDi3cAnGBV</t>
+          <t>Wtg8GXKfWxQjJGGYxmK7mUYTRcgSh9</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 450000000, "_seconds": 1712314609}</t>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>1712314609450</v>
+        <v>1706434207828</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>2.10.6</t>
+          <t>2.10.5</t>
         </is>
       </c>
       <c r="K102" t="n">
-        <v>6</v>
-      </c>
-      <c r="L102" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L102" t="n">
+        <v>80</v>
+      </c>
       <c r="M102" t="b">
         <v>0</v>
       </c>
       <c r="N102" t="n">
-        <v>-12</v>
+        <v>-4</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Gypsum (CaSO4)</t>
+          <t>Lactic Acid</t>
         </is>
       </c>
       <c r="Q102" t="b">
@@ -28247,7 +28249,7 @@
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T102" t="inlineStr">
@@ -28258,6 +28260,9 @@
       <c r="U102" t="b">
         <v>1</v>
       </c>
+      <c r="V102" t="inlineStr"/>
+      <c r="W102" t="inlineStr"/>
+      <c r="X102" t="inlineStr"/>
       <c r="Y102" t="inlineStr"/>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr"/>
@@ -28279,57 +28284,36 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>Wtg8GXKfWxQjJGGYxmK7mUYTRcgSh9</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
-        </is>
-      </c>
-      <c r="I103" t="n">
-        <v>1706434207828</v>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>2.10.5</t>
-        </is>
-      </c>
+          <t>default-6bc446</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
       <c r="K103" t="n">
-        <v>3</v>
-      </c>
-      <c r="L103" t="n">
-        <v>80</v>
-      </c>
-      <c r="M103" t="b">
-        <v>0</v>
-      </c>
-      <c r="N103" t="n">
-        <v>-4</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
-        </is>
+          <t>Biofine Clear</t>
+        </is>
+      </c>
+      <c r="P103" t="n">
+        <v>15</v>
       </c>
       <c r="Q103" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>Water Agent</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
@@ -28339,15 +28323,10 @@
       </c>
       <c r="T103" t="inlineStr">
         <is>
-          <t>Mash</t>
-        </is>
-      </c>
-      <c r="U103" t="b">
-        <v>1</v>
-      </c>
-      <c r="V103" t="inlineStr"/>
-      <c r="W103" t="inlineStr"/>
-      <c r="X103" t="inlineStr"/>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr"/>
       <c r="Y103" t="inlineStr"/>
       <c r="Z103" t="inlineStr"/>
       <c r="AA103" t="inlineStr"/>
@@ -28369,41 +28348,63 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>default-6bc446</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
+          <t>default-yn1j28sf</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>n9o5cFAQDFJBRKVV6LFjrQgK6Vnlsr</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 742000000, "_seconds": 1712314613}</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>1712314613742</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
       <c r="K104" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
+      <c r="M104" t="b">
+        <v>0</v>
+      </c>
+      <c r="N104" t="n">
+        <v>-11</v>
+      </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Biofine Clear</t>
+          <t>Yeast Nutrients</t>
         </is>
       </c>
       <c r="P104" t="n">
         <v>15</v>
       </c>
       <c r="Q104" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -28435,66 +28436,63 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+          <t>{"_nanoseconds": 538000000, "_seconds": 1697269076}</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>default-yn1j28sf</t>
+          <t>default-90c63c</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>n9o5cFAQDFJBRKVV6LFjrQgK6Vnlsr</t>
+          <t>n39qcIsSvY0mhj8mb0KhJHE9df0bXd</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 742000000, "_seconds": 1712314613}</t>
+          <t>{"_nanoseconds": 300000000, "_seconds": 1704369578}</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>1712314613742</v>
+        <v>1704369578300</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>2.10.6</t>
+          <t>2.10.4</t>
         </is>
       </c>
       <c r="K105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="b">
         <v>0</v>
       </c>
       <c r="N105" t="n">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>Yeast Nutrients</t>
-        </is>
-      </c>
-      <c r="P105" t="n">
-        <v>15</v>
+          <t>Gelatin</t>
+        </is>
       </c>
       <c r="Q105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
         <is>
-          <t>Boil</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="U105" t="inlineStr"/>
@@ -28506,12 +28504,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>First lager</t>
+          <t>Smash - Citra</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -28519,68 +28517,47 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 538000000, "_seconds": 1697269076}</t>
-        </is>
-      </c>
+      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>default-90c63c</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>n39qcIsSvY0mhj8mb0KhJHE9df0bXd</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 300000000, "_seconds": 1704369578}</t>
-        </is>
-      </c>
-      <c r="I106" t="n">
-        <v>1704369578300</v>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>2.10.4</t>
-        </is>
-      </c>
+          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
       <c r="K106" t="n">
-        <v>5</v>
+        <v>0.96</v>
       </c>
       <c r="L106" t="inlineStr"/>
-      <c r="M106" t="b">
-        <v>0</v>
-      </c>
-      <c r="N106" t="n">
-        <v>0</v>
-      </c>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Gelatin</t>
-        </is>
-      </c>
-      <c r="Q106" t="b">
-        <v>1</v>
-      </c>
+          <t>Calcium Chloride</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr"/>
       <c r="R106" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Water Agent</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T106" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Mash</t>
         </is>
       </c>
       <c r="U106" t="inlineStr"/>
+      <c r="V106" t="inlineStr"/>
+      <c r="W106" t="inlineStr"/>
+      <c r="X106" t="inlineStr"/>
       <c r="Y106" t="inlineStr"/>
       <c r="Z106" t="inlineStr"/>
       <c r="AA106" t="inlineStr"/>
@@ -28605,7 +28582,7 @@
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
+          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
@@ -28613,14 +28590,14 @@
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="n">
-        <v>0.96</v>
+        <v>10</v>
       </c>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Calcium Chloride</t>
+          <t>Epsom Salt (MgSO4)</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -28667,7 +28644,7 @@
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
+          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
@@ -28675,14 +28652,14 @@
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="n">
-        <v>10</v>
+        <v>17.64</v>
       </c>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Epsom Salt (MgSO4)</t>
+          <t>Gypsum (Calcium Sulfate)</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -28729,7 +28706,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
@@ -28737,17 +28714,21 @@
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="L109" t="inlineStr"/>
+        <v>20.8</v>
+      </c>
+      <c r="L109" t="n">
+        <v>80</v>
+      </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Gypsum (Calcium Sulfate)</t>
-        </is>
-      </c>
-      <c r="Q109" t="inlineStr"/>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q109" t="b">
+        <v>0</v>
+      </c>
       <c r="R109" t="inlineStr">
         <is>
           <t>Water Agent</t>
@@ -28755,7 +28736,7 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T109" t="inlineStr">
@@ -28763,7 +28744,9 @@
           <t>Mash</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr"/>
+      <c r="U109" t="b">
+        <v>1</v>
+      </c>
       <c r="V109" t="inlineStr"/>
       <c r="W109" t="inlineStr"/>
       <c r="X109" t="inlineStr"/>
@@ -28791,7 +28774,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
@@ -28799,21 +28782,17 @@
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="L110" t="n">
-        <v>80</v>
-      </c>
+        <v>2.9</v>
+      </c>
+      <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
-        </is>
-      </c>
-      <c r="Q110" t="b">
-        <v>0</v>
-      </c>
+          <t>Salt</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr"/>
       <c r="R110" t="inlineStr">
         <is>
           <t>Water Agent</t>
@@ -28821,7 +28800,7 @@
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T110" t="inlineStr">
@@ -28829,9 +28808,7 @@
           <t>Mash</t>
         </is>
       </c>
-      <c r="U110" t="b">
-        <v>1</v>
-      </c>
+      <c r="U110" t="inlineStr"/>
       <c r="V110" t="inlineStr"/>
       <c r="W110" t="inlineStr"/>
       <c r="X110" t="inlineStr"/>
@@ -28859,7 +28836,7 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
@@ -28867,17 +28844,21 @@
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="L111" t="inlineStr"/>
+        <v>3.05</v>
+      </c>
+      <c r="L111" t="n">
+        <v>80</v>
+      </c>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Salt</t>
-        </is>
-      </c>
-      <c r="Q111" t="inlineStr"/>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q111" t="b">
+        <v>0</v>
+      </c>
       <c r="R111" t="inlineStr">
         <is>
           <t>Water Agent</t>
@@ -28885,15 +28866,17 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T111" t="inlineStr">
         <is>
-          <t>Mash</t>
-        </is>
-      </c>
-      <c r="U111" t="inlineStr"/>
+          <t>Sparge</t>
+        </is>
+      </c>
+      <c r="U111" t="b">
+        <v>1</v>
+      </c>
       <c r="V111" t="inlineStr"/>
       <c r="W111" t="inlineStr"/>
       <c r="X111" t="inlineStr"/>
@@ -28921,7 +28904,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
@@ -28929,21 +28912,20 @@
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="L112" t="n">
-        <v>80</v>
-      </c>
+        <v>0.34</v>
+      </c>
+      <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
-        </is>
-      </c>
-      <c r="Q112" t="b">
-        <v>0</v>
-      </c>
+          <t>Calcium Chloride</t>
+        </is>
+      </c>
+      <c r="P112" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q112" t="inlineStr"/>
       <c r="R112" t="inlineStr">
         <is>
           <t>Water Agent</t>
@@ -28951,17 +28933,15 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T112" t="inlineStr">
         <is>
-          <t>Sparge</t>
-        </is>
-      </c>
-      <c r="U112" t="b">
-        <v>1</v>
-      </c>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr"/>
       <c r="V112" t="inlineStr"/>
       <c r="W112" t="inlineStr"/>
       <c r="X112" t="inlineStr"/>
@@ -28989,7 +28969,7 @@
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>new-ovmHGCc2JjuddQftQKRnRw2IqOPksF</t>
+          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
@@ -28997,14 +28977,14 @@
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="K113" t="n">
-        <v>0.34</v>
+        <v>3.62</v>
       </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Calcium Chloride</t>
+          <t>Epsom Salt (MgSO4)</t>
         </is>
       </c>
       <c r="P113" t="n">
@@ -29054,7 +29034,7 @@
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>new-tAM38RfHn8hFnmAABYZupbK1UzgFm1</t>
+          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
@@ -29062,14 +29042,14 @@
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="n">
-        <v>3.62</v>
+        <v>6.4</v>
       </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr"/>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Epsom Salt (MgSO4)</t>
+          <t>Gypsum (Calcium Sulfate)</t>
         </is>
       </c>
       <c r="P114" t="n">
@@ -29119,7 +29099,7 @@
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>new-yKxJxRIco7GpVVGCEKGJMSDpWPOLQm</t>
+          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
@@ -29127,14 +29107,14 @@
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
       <c r="K115" t="n">
-        <v>6.4</v>
+        <v>1.06</v>
       </c>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Gypsum (Calcium Sulfate)</t>
+          <t>Salt</t>
         </is>
       </c>
       <c r="P115" t="n">
@@ -29184,7 +29164,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>new-aOlKF4nejroi8r6Rz4mz7rBbuj7Ht3</t>
+          <t>new-TUfxqCta0ITj3uHT8vfAbVIfLtzqyA</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>
@@ -29192,28 +29172,28 @@
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
       <c r="K116" t="n">
-        <v>1.06</v>
+        <v>2</v>
       </c>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Salt</t>
+          <t>Protafloc</t>
         </is>
       </c>
       <c r="P116" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="Q116" t="inlineStr"/>
       <c r="R116" t="inlineStr">
         <is>
-          <t>Water Agent</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>tbsp</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -29249,7 +29229,7 @@
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>new-TUfxqCta0ITj3uHT8vfAbVIfLtzqyA</t>
+          <t>new-Xe5CxkyeaTwnbVay8pIU6ai8XycVKB</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
@@ -29264,7 +29244,7 @@
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Protafloc</t>
+          <t>Yeast Nutrient</t>
         </is>
       </c>
       <c r="P117" t="n">
@@ -29273,12 +29253,12 @@
       <c r="Q117" t="inlineStr"/>
       <c r="R117" t="inlineStr">
         <is>
-          <t>Fining</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>tbsp</t>
+          <t>tsp</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -29298,12 +29278,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Smash - Citra</t>
+          <t>Saison</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -29311,50 +29291,70 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>new-Xe5CxkyeaTwnbVay8pIU6ai8XycVKB</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
+          <t>default-2302b0</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>1781339599069</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
       <c r="K118" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
+      <c r="M118" t="b">
+        <v>0</v>
+      </c>
+      <c r="N118" t="n">
+        <v>94.5</v>
+      </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Yeast Nutrient</t>
-        </is>
-      </c>
-      <c r="P118" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q118" t="inlineStr"/>
+          <t>Baking Soda (NaHCO3)</t>
+        </is>
+      </c>
+      <c r="Q118" t="b">
+        <v>0</v>
+      </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Water Agent</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>tsp</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
         <is>
-          <t>Boil</t>
-        </is>
-      </c>
-      <c r="U118" t="inlineStr"/>
-      <c r="V118" t="inlineStr"/>
-      <c r="W118" t="inlineStr"/>
-      <c r="X118" t="inlineStr"/>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U118" t="b">
+        <v>1</v>
+      </c>
       <c r="Y118" t="inlineStr"/>
       <c r="Z118" t="inlineStr"/>
       <c r="AA118" t="inlineStr"/>
@@ -29378,26 +29378,26 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>default-2302b0</t>
+          <t>default-3b1827</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
         </is>
       </c>
       <c r="I119" t="n">
-        <v>1781339599069</v>
+        <v>1781339598782</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -29405,18 +29405,17 @@
         </is>
       </c>
       <c r="K119" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L119" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="M119" t="b">
         <v>0</v>
       </c>
       <c r="N119" t="n">
-        <v>94.5</v>
+        <v>44</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Baking Soda (NaHCO3)</t>
+          <t>Calcium Chloride (CaCl2)</t>
         </is>
       </c>
       <c r="Q119" t="b">
@@ -29463,44 +29462,45 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+          <t>{"_nanoseconds": 459000000, "_seconds": 1699176797}</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>default-3b1827</t>
+          <t>default-4e9d62</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>H7UJqQmCQoIgN0FnBDrWOqLcKcg5ej</t>
+          <t>baUPFv7WEZjl8hB5Cj0fMBSpkrFQ3R</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 782000000, "_seconds": 1781339598}</t>
+          <t>{"_nanoseconds": 229000000, "_seconds": 1704369577}</t>
         </is>
       </c>
       <c r="I120" t="n">
-        <v>1781339598782</v>
+        <v>1704369577229</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>3.0.1</t>
+          <t>2.10.4</t>
         </is>
       </c>
       <c r="K120" t="n">
         <v>2</v>
       </c>
+      <c r="L120" t="inlineStr"/>
       <c r="M120" t="b">
         <v>0</v>
       </c>
       <c r="N120" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Calcium Chloride (CaCl2)</t>
+          <t>Epsom Salt (MgSO4)</t>
         </is>
       </c>
       <c r="Q120" t="b">
@@ -29524,6 +29524,9 @@
       <c r="U120" t="b">
         <v>1</v>
       </c>
+      <c r="V120" t="inlineStr"/>
+      <c r="W120" t="inlineStr"/>
+      <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr"/>
       <c r="Z120" t="inlineStr"/>
       <c r="AA120" t="inlineStr"/>
@@ -29547,45 +29550,45 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 459000000, "_seconds": 1699176797}</t>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>default-4e9d62</t>
+          <t>default-1f88df</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>baUPFv7WEZjl8hB5Cj0fMBSpkrFQ3R</t>
+          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 229000000, "_seconds": 1704369577}</t>
+          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
         </is>
       </c>
       <c r="I121" t="n">
-        <v>1704369577229</v>
+        <v>1781339597373</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>2.10.4</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="b">
         <v>0</v>
       </c>
       <c r="N121" t="n">
-        <v>0</v>
+        <v>941.2</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Epsom Salt (MgSO4)</t>
+          <t>Gypsum (CaSO4)</t>
         </is>
       </c>
       <c r="Q121" t="b">
@@ -29609,9 +29612,6 @@
       <c r="U121" t="b">
         <v>1</v>
       </c>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr"/>
-      <c r="X121" t="inlineStr"/>
       <c r="Y121" t="inlineStr"/>
       <c r="Z121" t="inlineStr"/>
       <c r="AA121" t="inlineStr"/>
@@ -29635,26 +29635,26 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>default-1f88df</t>
+          <t>default-07adb1</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>NY07RRt0S89HR4jFBqrMhymNbPVBus</t>
+          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 373000000, "_seconds": 1781339597}</t>
+          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
         </is>
       </c>
       <c r="I122" t="n">
-        <v>1781339597373</v>
+        <v>1781339599470</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -29662,18 +29662,20 @@
         </is>
       </c>
       <c r="K122" t="n">
-        <v>3</v>
-      </c>
-      <c r="L122" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="L122" t="n">
+        <v>80</v>
+      </c>
       <c r="M122" t="b">
         <v>0</v>
       </c>
       <c r="N122" t="n">
-        <v>941.2</v>
+        <v>342.5</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>Gypsum (CaSO4)</t>
+          <t>Lactic Acid</t>
         </is>
       </c>
       <c r="Q122" t="b">
@@ -29686,7 +29688,7 @@
       </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="T122" t="inlineStr">
@@ -29720,26 +29722,26 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>default-07adb1</t>
+          <t>default-yn1j28sf</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>260vJiZ8NKF6Ccvlq0W1kKFJapTxCQ</t>
+          <t>92ChBNr2k0grfMSG7XIrynIVfyh02o</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 470000000, "_seconds": 1781339599}</t>
+          <t>{"_nanoseconds": 221000000, "_seconds": 1781339600}</t>
         </is>
       </c>
       <c r="I123" t="n">
-        <v>1781339599470</v>
+        <v>1781339600221</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -29747,43 +29749,42 @@
         </is>
       </c>
       <c r="K123" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L123" t="n">
-        <v>80</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L123" t="inlineStr"/>
       <c r="M123" t="b">
         <v>0</v>
       </c>
       <c r="N123" t="n">
-        <v>342.5</v>
+        <v>33</v>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Lactic Acid</t>
-        </is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P123" t="n">
+        <v>15</v>
       </c>
       <c r="Q123" t="b">
         <v>0</v>
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>Water Agent</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="S123" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="T123" t="inlineStr">
         <is>
-          <t>Mash</t>
-        </is>
-      </c>
-      <c r="U123" t="b">
-        <v>1</v>
-      </c>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr"/>
       <c r="Y123" t="inlineStr"/>
       <c r="Z123" t="inlineStr"/>
       <c r="AA123" t="inlineStr"/>
@@ -29807,26 +29808,26 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>default-yn1j28sf</t>
+          <t>default-5adf6e</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>92ChBNr2k0grfMSG7XIrynIVfyh02o</t>
+          <t>ntpZTYp6GFzhrk8IfC1bCJaKbHeIyI</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 221000000, "_seconds": 1781339600}</t>
+          <t>{"_nanoseconds": 65000000, "_seconds": 1778997170}</t>
         </is>
       </c>
       <c r="I124" t="n">
-        <v>1781339600221</v>
+        <v>1778997170065</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -29841,22 +29842,22 @@
         <v>0</v>
       </c>
       <c r="N124" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Yeast Nutrients</t>
+          <t>Irish Moss</t>
         </is>
       </c>
       <c r="P124" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q124" t="b">
         <v>0</v>
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Fining</t>
         </is>
       </c>
       <c r="S124" t="inlineStr">
@@ -29875,94 +29876,8 @@
       <c r="AA124" t="inlineStr"/>
       <c r="AB124" t="inlineStr"/>
     </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Saison</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>Misc</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>default-5adf6e</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>ntpZTYp6GFzhrk8IfC1bCJaKbHeIyI</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 65000000, "_seconds": 1778997170}</t>
-        </is>
-      </c>
-      <c r="I125" t="n">
-        <v>1778997170065</v>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>3.0.1</t>
-        </is>
-      </c>
-      <c r="K125" t="n">
-        <v>5</v>
-      </c>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="b">
-        <v>0</v>
-      </c>
-      <c r="N125" t="n">
-        <v>0</v>
-      </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>Irish Moss</t>
-        </is>
-      </c>
-      <c r="P125" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q125" t="b">
-        <v>0</v>
-      </c>
-      <c r="R125" t="inlineStr">
-        <is>
-          <t>Fining</t>
-        </is>
-      </c>
-      <c r="S125" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="T125" t="inlineStr">
-        <is>
-          <t>Boil</t>
-        </is>
-      </c>
-      <c r="U125" t="inlineStr"/>
-      <c r="Y125" t="inlineStr"/>
-      <c r="Z125" t="inlineStr"/>
-      <c r="AA125" t="inlineStr"/>
-      <c r="AB125" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AB125"/>
+  <autoFilter ref="A1:AB124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-08-01 05:25 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AO$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1900,8 +1900,75 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>American Pale Ale</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Ernst Gouws</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1.044619325</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1.009</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Repitch yeast
+Spund after 4 days
+Ferment on the cooler side 
+Not sure of the app's fg of 1.006 is realistic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P22"/>
+  <autoFilter ref="A1:P23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1912,7 +1979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT80"/>
+  <dimension ref="A1:AT81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10490,8 +10557,110 @@
       <c r="AS80" t="inlineStr"/>
       <c r="AT80" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>default-c3ff8bb88f9</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>BglUUy5uFFFvFjGd9EbIYIPvAJyyIE</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 508000000, "_seconds": 1785061181}</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>1785061181508</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Base (Pilsner)</t>
+        </is>
+      </c>
+      <c r="X81" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>Swaen Pilsner</t>
+        </is>
+      </c>
+      <c r="AE81" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF81" t="inlineStr"/>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH81" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI81" t="n">
+        <v>1.0368</v>
+      </c>
+      <c r="AJ81" t="n">
+        <v>80</v>
+      </c>
+      <c r="AL81" t="inlineStr"/>
+      <c r="AM81" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN81" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO81" t="inlineStr"/>
+      <c r="AP81" t="inlineStr"/>
+      <c r="AQ81" t="inlineStr"/>
+      <c r="AR81" t="inlineStr"/>
+      <c r="AS81" t="inlineStr"/>
+      <c r="AT81" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT80"/>
+  <autoFilter ref="A1:AT81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10502,7 +10671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO67"/>
+  <dimension ref="A1:AP71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10534,7 +10703,7 @@
     <col width="10" customWidth="1" min="27" max="27"/>
     <col width="11" customWidth="1" min="28" max="28"/>
     <col width="10" customWidth="1" min="29" max="29"/>
-    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
     <col width="11" customWidth="1" min="31" max="31"/>
     <col width="10" customWidth="1" min="32" max="32"/>
     <col width="53" customWidth="1" min="33" max="33"/>
@@ -10546,6 +10715,7 @@
     <col width="10" customWidth="1" min="39" max="39"/>
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="11" customWidth="1" min="41" max="41"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10752,6 +10922,11 @@
       <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>_editFlag</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>loss</t>
         </is>
       </c>
     </row>
@@ -10839,6 +11014,7 @@
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10944,6 +11120,7 @@
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11029,6 +11206,7 @@
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11114,6 +11292,7 @@
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11187,6 +11366,7 @@
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11260,6 +11440,7 @@
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11355,6 +11536,7 @@
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11450,6 +11632,7 @@
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11545,6 +11728,7 @@
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11654,6 +11838,7 @@
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11763,6 +11948,7 @@
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11872,6 +12058,7 @@
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11981,6 +12168,7 @@
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12090,6 +12278,7 @@
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12195,6 +12384,7 @@
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12303,6 +12493,7 @@
       <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12398,6 +12589,7 @@
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -12483,6 +12675,7 @@
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -12592,6 +12785,7 @@
       <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="inlineStr"/>
       <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -12701,6 +12895,7 @@
       <c r="AM21" t="inlineStr"/>
       <c r="AN21" t="inlineStr"/>
       <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12810,6 +13005,7 @@
       <c r="AM22" t="inlineStr"/>
       <c r="AN22" t="inlineStr"/>
       <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12919,6 +13115,7 @@
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13004,6 +13201,7 @@
       <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="inlineStr"/>
       <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13099,6 +13297,7 @@
       <c r="AM25" t="inlineStr"/>
       <c r="AN25" t="inlineStr"/>
       <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13207,6 +13406,7 @@
       <c r="AM26" t="inlineStr"/>
       <c r="AN26" t="inlineStr"/>
       <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13316,6 +13516,7 @@
       <c r="AM27" t="inlineStr"/>
       <c r="AN27" t="inlineStr"/>
       <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13425,6 +13626,7 @@
       <c r="AM28" t="inlineStr"/>
       <c r="AN28" t="inlineStr"/>
       <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13534,6 +13736,7 @@
       <c r="AM29" t="inlineStr"/>
       <c r="AN29" t="inlineStr"/>
       <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13629,6 +13832,7 @@
       <c r="AM30" t="inlineStr"/>
       <c r="AN30" t="inlineStr"/>
       <c r="AO30" t="inlineStr"/>
+      <c r="AP30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13724,6 +13928,7 @@
       <c r="AM31" t="inlineStr"/>
       <c r="AN31" t="inlineStr"/>
       <c r="AO31" t="inlineStr"/>
+      <c r="AP31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13832,6 +14037,7 @@
       </c>
       <c r="AN32" t="inlineStr"/>
       <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13937,6 +14143,7 @@
       <c r="AM33" t="inlineStr"/>
       <c r="AN33" t="inlineStr"/>
       <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14046,6 +14253,7 @@
       <c r="AM34" t="inlineStr"/>
       <c r="AN34" t="inlineStr"/>
       <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14159,6 +14367,7 @@
         <v>4</v>
       </c>
       <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14268,6 +14477,7 @@
         <v>4</v>
       </c>
       <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14353,6 +14563,7 @@
       <c r="AM37" t="inlineStr"/>
       <c r="AN37" t="inlineStr"/>
       <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14462,6 +14673,7 @@
       <c r="AM38" t="inlineStr"/>
       <c r="AN38" t="inlineStr"/>
       <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14557,6 +14769,7 @@
       <c r="AM39" t="inlineStr"/>
       <c r="AN39" t="inlineStr"/>
       <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14652,6 +14865,7 @@
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" t="inlineStr"/>
       <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14749,6 +14963,7 @@
       <c r="AM41" t="inlineStr"/>
       <c r="AN41" t="inlineStr"/>
       <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14844,6 +15059,7 @@
       <c r="AM42" t="inlineStr"/>
       <c r="AN42" t="inlineStr"/>
       <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14938,6 +15154,7 @@
       </c>
       <c r="AN43" t="inlineStr"/>
       <c r="AO43" t="inlineStr"/>
+      <c r="AP43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -15011,6 +15228,7 @@
       <c r="AM44" t="inlineStr"/>
       <c r="AN44" t="inlineStr"/>
       <c r="AO44" t="inlineStr"/>
+      <c r="AP44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -15106,6 +15324,7 @@
       <c r="AM45" t="inlineStr"/>
       <c r="AN45" t="inlineStr"/>
       <c r="AO45" t="inlineStr"/>
+      <c r="AP45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -15214,6 +15433,7 @@
       <c r="AM46" t="inlineStr"/>
       <c r="AN46" t="inlineStr"/>
       <c r="AO46" t="inlineStr"/>
+      <c r="AP46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -15287,6 +15507,7 @@
       <c r="AM47" t="inlineStr"/>
       <c r="AN47" t="inlineStr"/>
       <c r="AO47" t="inlineStr"/>
+      <c r="AP47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -15395,6 +15616,7 @@
       <c r="AM48" t="inlineStr"/>
       <c r="AN48" t="inlineStr"/>
       <c r="AO48" t="inlineStr"/>
+      <c r="AP48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15493,6 +15715,7 @@
       <c r="AM49" t="inlineStr"/>
       <c r="AN49" t="inlineStr"/>
       <c r="AO49" t="inlineStr"/>
+      <c r="AP49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15566,6 +15789,7 @@
       <c r="AM50" t="inlineStr"/>
       <c r="AN50" t="inlineStr"/>
       <c r="AO50" t="inlineStr"/>
+      <c r="AP50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15641,6 +15865,7 @@
       <c r="AL51" t="inlineStr"/>
       <c r="AN51" t="inlineStr"/>
       <c r="AO51" t="inlineStr"/>
+      <c r="AP51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15716,6 +15941,7 @@
       <c r="AL52" t="inlineStr"/>
       <c r="AN52" t="inlineStr"/>
       <c r="AO52" t="inlineStr"/>
+      <c r="AP52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15824,6 +16050,7 @@
       <c r="AM53" t="inlineStr"/>
       <c r="AN53" t="inlineStr"/>
       <c r="AO53" t="inlineStr"/>
+      <c r="AP53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15897,6 +16124,7 @@
       <c r="AM54" t="inlineStr"/>
       <c r="AN54" t="inlineStr"/>
       <c r="AO54" t="inlineStr"/>
+      <c r="AP54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15970,6 +16198,7 @@
       <c r="AM55" t="inlineStr"/>
       <c r="AN55" t="inlineStr"/>
       <c r="AO55" t="inlineStr"/>
+      <c r="AP55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -16045,6 +16274,7 @@
       <c r="AL56" t="inlineStr"/>
       <c r="AN56" t="inlineStr"/>
       <c r="AO56" t="inlineStr"/>
+      <c r="AP56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -16120,6 +16350,7 @@
       <c r="AL57" t="inlineStr"/>
       <c r="AN57" t="inlineStr"/>
       <c r="AO57" t="inlineStr"/>
+      <c r="AP57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -16193,6 +16424,7 @@
       <c r="AM58" t="inlineStr"/>
       <c r="AN58" t="inlineStr"/>
       <c r="AO58" t="inlineStr"/>
+      <c r="AP58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -16266,6 +16498,7 @@
       <c r="AM59" t="inlineStr"/>
       <c r="AN59" t="inlineStr"/>
       <c r="AO59" t="inlineStr"/>
+      <c r="AP59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16349,6 +16582,7 @@
       <c r="AO60" t="b">
         <v>1</v>
       </c>
+      <c r="AP60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16430,6 +16664,7 @@
       <c r="AM61" t="inlineStr"/>
       <c r="AN61" t="inlineStr"/>
       <c r="AO61" t="inlineStr"/>
+      <c r="AP61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16511,6 +16746,7 @@
       <c r="AM62" t="inlineStr"/>
       <c r="AN62" t="inlineStr"/>
       <c r="AO62" t="inlineStr"/>
+      <c r="AP62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -16592,6 +16828,7 @@
       <c r="AM63" t="inlineStr"/>
       <c r="AN63" t="inlineStr"/>
       <c r="AO63" t="inlineStr"/>
+      <c r="AP63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -16680,6 +16917,7 @@
       <c r="AO64" t="b">
         <v>1</v>
       </c>
+      <c r="AP64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -16797,6 +17035,7 @@
       <c r="AM65" t="inlineStr"/>
       <c r="AN65" t="inlineStr"/>
       <c r="AO65" t="inlineStr"/>
+      <c r="AP65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -16905,6 +17144,7 @@
       <c r="AM66" t="inlineStr"/>
       <c r="AN66" t="inlineStr"/>
       <c r="AO66" t="inlineStr"/>
+      <c r="AP66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -17022,9 +17262,428 @@
       <c r="AM67" t="inlineStr"/>
       <c r="AN67" t="inlineStr"/>
       <c r="AO67" t="inlineStr"/>
+      <c r="AP67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H68" t="n">
+        <v>5</v>
+      </c>
+      <c r="J68" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N68" t="b">
+        <v>0</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="S68" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z68" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr"/>
+      <c r="AG68" t="inlineStr"/>
+      <c r="AH68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr"/>
+      <c r="AJ68" t="inlineStr"/>
+      <c r="AK68" t="inlineStr"/>
+      <c r="AL68" t="inlineStr"/>
+      <c r="AM68" t="inlineStr"/>
+      <c r="AN68" t="inlineStr"/>
+      <c r="AO68" t="inlineStr"/>
+      <c r="AP68" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H69" t="n">
+        <v>10</v>
+      </c>
+      <c r="J69" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N69" t="b">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="S69" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z69" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AG69" t="inlineStr"/>
+      <c r="AH69" t="inlineStr"/>
+      <c r="AI69" t="inlineStr"/>
+      <c r="AJ69" t="inlineStr"/>
+      <c r="AK69" t="inlineStr"/>
+      <c r="AL69" t="inlineStr"/>
+      <c r="AM69" t="inlineStr"/>
+      <c r="AN69" t="inlineStr"/>
+      <c r="AO69" t="inlineStr"/>
+      <c r="AP69" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H70" t="n">
+        <v>25</v>
+      </c>
+      <c r="J70" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N70" t="b">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="S70" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr"/>
+      <c r="AJ70" t="inlineStr"/>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="inlineStr"/>
+      <c r="AM70" t="inlineStr"/>
+      <c r="AN70" t="inlineStr"/>
+      <c r="AO70" t="inlineStr"/>
+      <c r="AP70" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H71" t="n">
+        <v>40</v>
+      </c>
+      <c r="J71" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N71" t="b">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="S71" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Y71" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AG71" t="inlineStr"/>
+      <c r="AH71" t="inlineStr"/>
+      <c r="AI71" t="inlineStr"/>
+      <c r="AJ71" t="inlineStr"/>
+      <c r="AK71" t="inlineStr"/>
+      <c r="AL71" t="inlineStr"/>
+      <c r="AN71" t="inlineStr"/>
+      <c r="AO71" t="inlineStr"/>
+      <c r="AP71" t="n">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO67"/>
+  <autoFilter ref="A1:AP71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17035,7 +17694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL22"/>
+  <dimension ref="A1:AL23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19520,8 +20179,131 @@
         <v>1</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>default-qytQJkV9cQwX6g1aZ4Carqa9z0LXeE</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>250</v>
+      </c>
+      <c r="H23" t="n">
+        <v>80</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Medium-Low</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>WHC Lab</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>13</v>
+      </c>
+      <c r="R23" t="n">
+        <v>80</v>
+      </c>
+      <c r="S23" t="n">
+        <v>22</v>
+      </c>
+      <c r="T23" t="n">
+        <v>76</v>
+      </c>
+      <c r="U23" t="n">
+        <v>18</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Clean West Coast IPA</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>LAX</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Repitch</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 443000000, "_seconds": 1784057955}</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>7L5ixnuXBXaqmTBXyQnlfKg5wkjOhb</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 72000000, "_seconds": 1785061190}</t>
+        </is>
+      </c>
+      <c r="AJ23" t="n">
+        <v>1785061190072</v>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL23" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL22"/>
+  <autoFilter ref="A1:AL23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19532,7 +20314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB124"/>
+  <dimension ref="A1:AB129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -29876,8 +30658,436 @@
       <c r="AA124" t="inlineStr"/>
       <c r="AB124" t="inlineStr"/>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>default-3b1827</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Krt6pCjgS31xUqPji18XahSkMlPSpg</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 542000000, "_seconds": 1785061186}</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>1785061186542</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>2</v>
+      </c>
+      <c r="M125" t="b">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Calcium Chloride (CaCl2)</t>
+        </is>
+      </c>
+      <c r="Q125" t="b">
+        <v>0</v>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U125" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y125" t="inlineStr"/>
+      <c r="Z125" t="inlineStr"/>
+      <c r="AA125" t="inlineStr"/>
+      <c r="AB125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>default-1f88df</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>1eZxGCR6vlM3Yk5utOhCaPxCJgad8G</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 868000000, "_seconds": 1785061185}</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>1785061185868</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>3</v>
+      </c>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="b">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>936.7</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Gypsum (CaSO4)</t>
+        </is>
+      </c>
+      <c r="Q126" t="b">
+        <v>0</v>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U126" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y126" t="inlineStr"/>
+      <c r="Z126" t="inlineStr"/>
+      <c r="AA126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2K0l0yVaTOoSGIybTyu7f2OZzHqTjY</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 167000000, "_seconds": 1785061187}</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>1785061187167</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>2</v>
+      </c>
+      <c r="L127" t="n">
+        <v>80</v>
+      </c>
+      <c r="M127" t="b">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>340.5</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q127" t="b">
+        <v>0</v>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U127" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y127" t="inlineStr"/>
+      <c r="Z127" t="inlineStr"/>
+      <c r="AA127" t="inlineStr"/>
+      <c r="AB127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>default-yn1j28sf</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>92ChBNr2k0grfMSG7XIrynIVfyh02o</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 221000000, "_seconds": 1781339600}</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>1781339600221</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>1</v>
+      </c>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="b">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
+        <v>33</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P128" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q128" t="b">
+        <v>0</v>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr"/>
+      <c r="Y128" t="inlineStr"/>
+      <c r="Z128" t="inlineStr"/>
+      <c r="AA128" t="inlineStr"/>
+      <c r="AB128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Smash Mosaic</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>default-5adf6e</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>hBAibaPvX0FHQT9ll1gxER4gHbbxIg</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1785061187}</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>1785061187983</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>1</v>
+      </c>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="b">
+        <v>0</v>
+      </c>
+      <c r="N129" t="n">
+        <v>-5</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Irish Moss</t>
+        </is>
+      </c>
+      <c r="P129" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q129" t="b">
+        <v>0</v>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr"/>
+      <c r="Y129" t="inlineStr"/>
+      <c r="Z129" t="inlineStr"/>
+      <c r="AA129" t="inlineStr"/>
+      <c r="AB129" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB124"/>
+  <autoFilter ref="A1:AB129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-08-05 05:12 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1962,13 +1962,78 @@
         <is>
           <t>Repitch yeast
 Spund after 4 days
-Ferment on the cooler side 
 Not sure of the app's fg of 1.006 is realistic</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>American Pale Ale</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ernst Gouws</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1.044619325</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1.007</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Repitch yeast
+Spund after 4 days
+Not sure of the app's fg of 1.006 is realistic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P23"/>
+  <autoFilter ref="A1:P24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1979,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT83"/>
+  <dimension ref="A1:AT84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10903,8 +10968,110 @@
       <c r="AS83" t="inlineStr"/>
       <c r="AT83" t="inlineStr"/>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>default-c3ff8bb88f9</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>BglUUy5uFFFvFjGd9EbIYIPvAJyyIE</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 508000000, "_seconds": 1785061181}</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>1785061181508</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>Base (Pilsner)</t>
+        </is>
+      </c>
+      <c r="X84" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z84" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>Swaen Pilsner</t>
+        </is>
+      </c>
+      <c r="AE84" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF84" t="inlineStr"/>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH84" t="n">
+        <v>100</v>
+      </c>
+      <c r="AI84" t="n">
+        <v>1.0368</v>
+      </c>
+      <c r="AJ84" t="n">
+        <v>80</v>
+      </c>
+      <c r="AL84" t="inlineStr"/>
+      <c r="AM84" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN84" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO84" t="inlineStr"/>
+      <c r="AP84" t="inlineStr"/>
+      <c r="AQ84" t="inlineStr"/>
+      <c r="AR84" t="inlineStr"/>
+      <c r="AS84" t="inlineStr"/>
+      <c r="AT84" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT83"/>
+  <autoFilter ref="A1:AT84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10915,7 +11082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP72"/>
+  <dimension ref="A1:AP76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18096,8 +18263,506 @@
         <v>15</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H73" t="n">
+        <v>11</v>
+      </c>
+      <c r="J73" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N73" t="b">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="S73" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z73" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB73" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr"/>
+      <c r="AG73" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AH73" t="inlineStr">
+        <is>
+          <t>LISH4vcmJYasu0xkwyZMJ3hK9ZNvds</t>
+        </is>
+      </c>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AJ73" t="n">
+        <v>1785754354406</v>
+      </c>
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL73" t="n">
+        <v>200</v>
+      </c>
+      <c r="AM73" t="inlineStr"/>
+      <c r="AN73" t="inlineStr"/>
+      <c r="AO73" t="inlineStr"/>
+      <c r="AP73" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H74" t="n">
+        <v>10</v>
+      </c>
+      <c r="J74" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N74" t="b">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="S74" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z74" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB74" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AG74" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AH74" t="inlineStr">
+        <is>
+          <t>LISH4vcmJYasu0xkwyZMJ3hK9ZNvds</t>
+        </is>
+      </c>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AJ74" t="n">
+        <v>1785754354406</v>
+      </c>
+      <c r="AK74" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL74" t="n">
+        <v>200</v>
+      </c>
+      <c r="AM74" t="inlineStr"/>
+      <c r="AN74" t="inlineStr"/>
+      <c r="AO74" t="inlineStr"/>
+      <c r="AP74" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>25</v>
+      </c>
+      <c r="J75" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N75" t="b">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="S75" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Z75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB75" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AH75" t="inlineStr">
+        <is>
+          <t>LISH4vcmJYasu0xkwyZMJ3hK9ZNvds</t>
+        </is>
+      </c>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AJ75" t="n">
+        <v>1785754354406</v>
+      </c>
+      <c r="AK75" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL75" t="n">
+        <v>200</v>
+      </c>
+      <c r="AM75" t="inlineStr"/>
+      <c r="AN75" t="inlineStr"/>
+      <c r="AO75" t="inlineStr"/>
+      <c r="AP75" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>default-0c4aeb7c</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H76" t="n">
+        <v>40</v>
+      </c>
+      <c r="J76" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N76" t="b">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="S76" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Mosaic</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>Citra®</t>
+        </is>
+      </c>
+      <c r="Y76" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB76" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>India Pale Ale, Pale Ale</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AG76" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>LISH4vcmJYasu0xkwyZMJ3hK9ZNvds</t>
+        </is>
+      </c>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 406000000, "_seconds": 1785754354}</t>
+        </is>
+      </c>
+      <c r="AJ76" t="n">
+        <v>1785754354406</v>
+      </c>
+      <c r="AK76" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL76" t="n">
+        <v>200</v>
+      </c>
+      <c r="AN76" t="inlineStr"/>
+      <c r="AO76" t="inlineStr"/>
+      <c r="AP76" t="n">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AP72"/>
+  <autoFilter ref="A1:AP76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18108,7 +18773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL23"/>
+  <dimension ref="A1:AL24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -20716,8 +21381,131 @@
         <v>0</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>default-qytQJkV9cQwX6g1aZ4Carqa9z0LXeE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>250</v>
+      </c>
+      <c r="H24" t="n">
+        <v>80</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Medium-Low</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>WHC Lab</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>13</v>
+      </c>
+      <c r="R24" t="n">
+        <v>80</v>
+      </c>
+      <c r="S24" t="n">
+        <v>22</v>
+      </c>
+      <c r="T24" t="n">
+        <v>76</v>
+      </c>
+      <c r="U24" t="n">
+        <v>18</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Clean West Coast IPA</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>LAX</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Repitch</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 443000000, "_seconds": 1784057955}</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>7L5ixnuXBXaqmTBXyQnlfKg5wkjOhb</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 72000000, "_seconds": 1785061190}</t>
+        </is>
+      </c>
+      <c r="AJ24" t="n">
+        <v>1785061190072</v>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL23"/>
+  <autoFilter ref="A1:AL24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20728,7 +21516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB129"/>
+  <dimension ref="A1:AB134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -31500,8 +32288,436 @@
       <c r="AA129" t="inlineStr"/>
       <c r="AB129" t="inlineStr"/>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>default-3b1827</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Krt6pCjgS31xUqPji18XahSkMlPSpg</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 542000000, "_seconds": 1785061186}</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>1785061186542</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>2</v>
+      </c>
+      <c r="M130" t="b">
+        <v>0</v>
+      </c>
+      <c r="N130" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Calcium Chloride (CaCl2)</t>
+        </is>
+      </c>
+      <c r="Q130" t="b">
+        <v>0</v>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U130" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y130" t="inlineStr"/>
+      <c r="Z130" t="inlineStr"/>
+      <c r="AA130" t="inlineStr"/>
+      <c r="AB130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>default-1f88df</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>1eZxGCR6vlM3Yk5utOhCaPxCJgad8G</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 868000000, "_seconds": 1785061185}</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>1785061185868</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>3</v>
+      </c>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="b">
+        <v>0</v>
+      </c>
+      <c r="N131" t="n">
+        <v>936.7</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Gypsum (CaSO4)</t>
+        </is>
+      </c>
+      <c r="Q131" t="b">
+        <v>0</v>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U131" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y131" t="inlineStr"/>
+      <c r="Z131" t="inlineStr"/>
+      <c r="AA131" t="inlineStr"/>
+      <c r="AB131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2K0l0yVaTOoSGIybTyu7f2OZzHqTjY</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 167000000, "_seconds": 1785061187}</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>1785061187167</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>2</v>
+      </c>
+      <c r="L132" t="n">
+        <v>80</v>
+      </c>
+      <c r="M132" t="b">
+        <v>0</v>
+      </c>
+      <c r="N132" t="n">
+        <v>340.5</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q132" t="b">
+        <v>0</v>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U132" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y132" t="inlineStr"/>
+      <c r="Z132" t="inlineStr"/>
+      <c r="AA132" t="inlineStr"/>
+      <c r="AB132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>default-yn1j28sf</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>92ChBNr2k0grfMSG7XIrynIVfyh02o</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 221000000, "_seconds": 1781339600}</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>1781339600221</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>1</v>
+      </c>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="b">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>33</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P133" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q133" t="b">
+        <v>0</v>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr"/>
+      <c r="Y133" t="inlineStr"/>
+      <c r="Z133" t="inlineStr"/>
+      <c r="AA133" t="inlineStr"/>
+      <c r="AB133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Smash shoddy</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 504000000, "_seconds": 1775809151}</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>default-5adf6e</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>hBAibaPvX0FHQT9ll1gxER4gHbbxIg</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1785061187}</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>1785061187983</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K134" t="n">
+        <v>1</v>
+      </c>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="b">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>-5</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>Irish Moss</t>
+        </is>
+      </c>
+      <c r="P134" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q134" t="b">
+        <v>0</v>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr"/>
+      <c r="Y134" t="inlineStr"/>
+      <c r="Z134" t="inlineStr"/>
+      <c r="AA134" t="inlineStr"/>
+      <c r="AB134" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB129"/>
+  <autoFilter ref="A1:AB134"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: 2026-08-06 05:14 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -1941,7 +1941,7 @@
         <v>4.99</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>34.9</v>
+        <v>36.6</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>3.4</v>
@@ -18162,7 +18162,7 @@
         <v>11.1</v>
       </c>
       <c r="H72" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="J72" t="n">
         <v>5.6</v>
@@ -18180,7 +18180,7 @@
         <v>0.1</v>
       </c>
       <c r="Q72" t="n">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="S72" t="n">
         <v>40.6</v>

</xml_diff>

<commit_message>
Update: 2026-08-15 02:49 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -1935,13 +1935,13 @@
         <v>1.044619325</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>1.007</v>
+        <v>1.006</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>4.99</v>
+        <v>5.12</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>36.6</v>
+        <v>37.7</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>3.4</v>
@@ -18038,7 +18038,7 @@
         <v>11.1</v>
       </c>
       <c r="H71" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="J71" t="n">
         <v>5.6</v>
@@ -18056,7 +18056,7 @@
         <v>0.1</v>
       </c>
       <c r="Q71" t="n">
-        <v>4.3</v>
+        <v>5.1</v>
       </c>
       <c r="S71" t="n">
         <v>40.6</v>
@@ -18162,7 +18162,7 @@
         <v>11.1</v>
       </c>
       <c r="H72" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J72" t="n">
         <v>5.6</v>
@@ -18180,7 +18180,7 @@
         <v>0.1</v>
       </c>
       <c r="Q72" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="S72" t="n">
         <v>40.6</v>
@@ -31989,7 +31989,7 @@
         </is>
       </c>
       <c r="K126" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="b">

</xml_diff>

<commit_message>
Update: 2026-08-16 02:56 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -1941,7 +1941,7 @@
         <v>5.12</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="K23" s="4" t="n">
         <v>3.4</v>
@@ -18038,7 +18038,7 @@
         <v>11.1</v>
       </c>
       <c r="H71" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J71" t="n">
         <v>5.6</v>
@@ -18056,7 +18056,7 @@
         <v>0.1</v>
       </c>
       <c r="Q71" t="n">
-        <v>5.1</v>
+        <v>5.5</v>
       </c>
       <c r="S71" t="n">
         <v>40.6</v>
@@ -18162,7 +18162,7 @@
         <v>11.1</v>
       </c>
       <c r="H72" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J72" t="n">
         <v>5.6</v>
@@ -18180,7 +18180,7 @@
         <v>0.1</v>
       </c>
       <c r="Q72" t="n">
-        <v>8.800000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="S72" t="n">
         <v>40.6</v>

</xml_diff>

<commit_message>
Update: 2026-09-03 06:49 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$140</definedName>
@@ -2080,7 +2080,7 @@
         <v>22.7</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>12</v>
@@ -2108,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT87"/>
+  <dimension ref="A1:AT86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11024,26 +11024,26 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 218000000, "_seconds": 1784057842}</t>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>default-c4dd41c950d</t>
+          <t>default-c3ff8bb88f9</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>AXp7oOluCAHfEYcypMwZBoIFWG2sY2</t>
+          <t>GOG6rzO2xrYYSto1fMsaU5lUVzV9v7</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 217000000, "_seconds": 1784057842}</t>
+          <t>{"_nanoseconds": 7000000, "_seconds": 1786789728}</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>1784057842217</v>
+        <v>1786789728007</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -11051,10 +11051,10 @@
         </is>
       </c>
       <c r="L84" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="Q84" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="W84" t="inlineStr">
         <is>
@@ -11065,11 +11065,11 @@
         <v>0</v>
       </c>
       <c r="Z84" t="n">
-        <v>2</v>
+        <v>11.4</v>
       </c>
       <c r="AD84" t="inlineStr">
         <is>
-          <t>Swaen Lager</t>
+          <t>Swaen Pilsner</t>
         </is>
       </c>
       <c r="AE84" t="b">
@@ -11082,7 +11082,7 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>62.5</v>
+        <v>78.13</v>
       </c>
       <c r="AI84" t="n">
         <v>1.0368</v>
@@ -11126,26 +11126,26 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>default-c3ff8bb88f9</t>
+          <t>default-d9e04639a2c</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>GOG6rzO2xrYYSto1fMsaU5lUVzV9v7</t>
+          <t>vNwfSmBlJ1e4z5jdNJOlLtSxOILZid</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 7000000, "_seconds": 1786789728}</t>
+          <t>{"_nanoseconds": 15000000, "_seconds": 1785061182}</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>1786789728007</v>
+        <v>1785061182015</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -11156,22 +11156,22 @@
         <v>0.5</v>
       </c>
       <c r="Q85" t="n">
-        <v>1.9</v>
+        <v>5.1</v>
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>Base (Pilsner)</t>
+          <t>Base (Vienna)</t>
         </is>
       </c>
       <c r="X85" t="b">
         <v>0</v>
       </c>
       <c r="Z85" t="n">
-        <v>11.4</v>
+        <v>2.4</v>
       </c>
       <c r="AD85" t="inlineStr">
         <is>
-          <t>Swaen Pilsner</t>
+          <t>Swaen Vienna</t>
         </is>
       </c>
       <c r="AE85" t="b">
@@ -11187,10 +11187,10 @@
         <v>15.63</v>
       </c>
       <c r="AI85" t="n">
-        <v>1.0368</v>
+        <v>1.03588</v>
       </c>
       <c r="AJ85" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AL85" t="inlineStr"/>
       <c r="AM85" t="inlineStr">
@@ -11226,78 +11226,83 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>default-d9e04639a2c</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>vNwfSmBlJ1e4z5jdNJOlLtSxOILZid</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 15000000, "_seconds": 1785061182}</t>
-        </is>
-      </c>
-      <c r="I86" t="n">
-        <v>1785061182015</v>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>3.0.1</t>
-        </is>
+          <t>default-MSMYXD2BJLGqRAHlZVbqdHLIa0VzoF</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="n">
+        <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="P86" t="n">
+        <v>1.5</v>
       </c>
       <c r="Q86" t="n">
-        <v>5.1</v>
+        <v>2.5380711</v>
+      </c>
+      <c r="S86" t="n">
+        <v>0</v>
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>Base (Vienna)</t>
+          <t>Base (Wheat)</t>
         </is>
       </c>
       <c r="X86" t="b">
         <v>0</v>
       </c>
-      <c r="Z86" t="n">
-        <v>2.4</v>
+      <c r="Y86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB86" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>10</v>
       </c>
       <c r="AD86" t="inlineStr">
         <is>
-          <t>Swaen Vienna</t>
+          <t>Torrefied Wheat</t>
         </is>
       </c>
       <c r="AE86" t="b">
         <v>0</v>
       </c>
-      <c r="AF86" t="inlineStr"/>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>Pre-cooked, non-malted cereals provide the brewer with the opportunity for product differentiation. Flaked products can be added directly to the mash without the need for milling.</t>
+        </is>
+      </c>
       <c r="AG86" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>15.63</v>
+        <v>6.25</v>
       </c>
       <c r="AI86" t="n">
-        <v>1.03588</v>
+        <v>1.038</v>
       </c>
       <c r="AJ86" t="n">
-        <v>78</v>
+        <v>82</v>
+      </c>
+      <c r="AK86" t="n">
+        <v>10</v>
       </c>
       <c r="AL86" t="inlineStr"/>
       <c r="AM86" t="inlineStr">
         <is>
-          <t>The Swaen</t>
+          <t>Crisp</t>
         </is>
       </c>
       <c r="AN86" t="inlineStr">
@@ -11312,115 +11317,8 @@
       <c r="AS86" t="inlineStr"/>
       <c r="AT86" t="inlineStr"/>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>TtkyFZuS1krih6K7d2BW7nY3qFmYPZ</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Kalahari blond</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Fermentable</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>default-MSMYXD2BJLGqRAHlZVbqdHLIa0VzoF</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="n">
-        <v>0</v>
-      </c>
-      <c r="L87" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M87" t="inlineStr"/>
-      <c r="P87" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Q87" t="n">
-        <v>2.5380711</v>
-      </c>
-      <c r="S87" t="n">
-        <v>0</v>
-      </c>
-      <c r="W87" t="inlineStr">
-        <is>
-          <t>Base (Wheat)</t>
-        </is>
-      </c>
-      <c r="X87" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y87" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB87" t="n">
-        <v>25</v>
-      </c>
-      <c r="AC87" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD87" t="inlineStr">
-        <is>
-          <t>Torrefied Wheat</t>
-        </is>
-      </c>
-      <c r="AE87" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF87" t="inlineStr">
-        <is>
-          <t>Pre-cooked, non-malted cereals provide the brewer with the opportunity for product differentiation. Flaked products can be added directly to the mash without the need for milling.</t>
-        </is>
-      </c>
-      <c r="AG87" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="AH87" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="AI87" t="n">
-        <v>1.038</v>
-      </c>
-      <c r="AJ87" t="n">
-        <v>82</v>
-      </c>
-      <c r="AK87" t="n">
-        <v>10</v>
-      </c>
-      <c r="AL87" t="inlineStr"/>
-      <c r="AM87" t="inlineStr">
-        <is>
-          <t>Crisp</t>
-        </is>
-      </c>
-      <c r="AN87" t="inlineStr">
-        <is>
-          <t>Grain</t>
-        </is>
-      </c>
-      <c r="AO87" t="inlineStr"/>
-      <c r="AP87" t="inlineStr"/>
-      <c r="AQ87" t="inlineStr"/>
-      <c r="AR87" t="inlineStr"/>
-      <c r="AS87" t="inlineStr"/>
-      <c r="AT87" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AT87"/>
+  <autoFilter ref="A1:AT86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update: 2026-09-09 07:02 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1.047482398</v>
+        <v>1.046512226</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>1.008</v>
@@ -2077,19 +2077,19 @@
         <v>5.12</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>22.7</v>
+        <v>22.2</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>18.6</v>
+        <v>22.77</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>57.9</v>
+        <v>60.5</v>
       </c>
       <c r="O25" s="3" t="n">
         <v>70</v>
@@ -11014,7 +11014,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -11051,7 +11051,7 @@
         </is>
       </c>
       <c r="L84" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="Q84" t="n">
         <v>1.9</v>
@@ -11082,7 +11082,7 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>78.13</v>
+        <v>77.5</v>
       </c>
       <c r="AI84" t="n">
         <v>1.0368</v>
@@ -11116,7 +11116,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -11153,7 +11153,7 @@
         </is>
       </c>
       <c r="L85" t="n">
-        <v>0.5</v>
+        <v>0.64</v>
       </c>
       <c r="Q85" t="n">
         <v>5.1</v>
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="AH85" t="n">
-        <v>15.63</v>
+        <v>16</v>
       </c>
       <c r="AI85" t="n">
         <v>1.03588</v>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -11240,7 +11240,7 @@
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="P86" t="n">
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="AI86" t="n">
         <v>1.038</v>
@@ -19018,7 +19018,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -19035,7 +19035,7 @@
         <v>6.3</v>
       </c>
       <c r="H77" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J77" t="n">
         <v>3.5</v>
@@ -19047,7 +19047,7 @@
         <v>30</v>
       </c>
       <c r="Q77" t="n">
-        <v>16.6</v>
+        <v>15.6</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -19127,7 +19127,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -19144,13 +19144,13 @@
         <v>3.2</v>
       </c>
       <c r="H78" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N78" t="b">
         <v>0</v>
       </c>
       <c r="Q78" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -19225,7 +19225,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -19242,13 +19242,13 @@
         <v>3.2</v>
       </c>
       <c r="H79" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N79" t="b">
         <v>0</v>
       </c>
       <c r="Q79" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -22068,7 +22068,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -33473,7 +33473,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -33510,7 +33510,7 @@
         </is>
       </c>
       <c r="K136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M136" t="b">
         <v>0</v>
@@ -33557,7 +33557,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -33594,7 +33594,7 @@
         </is>
       </c>
       <c r="K137" t="n">
-        <v>2</v>
+        <v>2.667</v>
       </c>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="b">
@@ -33642,7 +33642,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -33679,7 +33679,7 @@
         </is>
       </c>
       <c r="K138" t="n">
-        <v>2</v>
+        <v>2.667</v>
       </c>
       <c r="L138" t="n">
         <v>80</v>
@@ -33729,7 +33729,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -33766,7 +33766,7 @@
         </is>
       </c>
       <c r="K139" t="n">
-        <v>5</v>
+        <v>6.667</v>
       </c>
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="b">
@@ -33815,7 +33815,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Kalahari blond</t>
+          <t>Kalahari blond 16 liter</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -33852,7 +33852,7 @@
         </is>
       </c>
       <c r="K140" t="n">
-        <v>0.76</v>
+        <v>1.013</v>
       </c>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="b">

</xml_diff>

<commit_message>
Update: 2026-09-12 06:49 SAST
</commit_message>
<xml_diff>
--- a/exports/Brewfather_Recipes_Summary.xlsx
+++ b/exports/Brewfather_Recipes_Summary.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$86</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recipes'!$A$1:$P$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fermentables'!$A$1:$AT$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hops'!$A$1:$AP$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Yeast'!$A$1:$AL$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Misc'!$A$1:$AB$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1674,19 +1674,19 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1.048764437</v>
+        <v>1.047685263</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>1.009</v>
+        <v>1.01</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>5.25</v>
+        <v>4.99</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>33.1</v>
+        <v>30.3</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>12</v>
@@ -1708,8 +1708,7 @@
 Larger portion pilsener malt
 Used American Pale Ale water profile 
 V2 with lax came out more like a blonde.
-For v3
-less malty (drop vienna) and even more whirlpool hops.</t>
+Future: less malty (drop vienna) and even more whirlpool hops.</t>
         </is>
       </c>
     </row>
@@ -2068,19 +2067,19 @@
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1.046512226</v>
+        <v>1.0454136</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>1.008</v>
+        <v>1.007</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>5.12</v>
+        <v>4.99</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>16</v>
@@ -2096,8 +2095,72 @@
       </c>
       <c r="P25" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>English Porter</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>All Grain</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ernst Gouws</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>1.047801523</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Dryer summer stout with whc heritage yeast.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P25"/>
+  <autoFilter ref="A1:P26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2108,7 +2171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT86"/>
+  <dimension ref="A1:AT93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2127,7 +2190,7 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
@@ -9553,7 +9616,7 @@
         </is>
       </c>
       <c r="L70" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="Q70" t="n">
         <v>1.9</v>
@@ -9584,7 +9647,7 @@
         </is>
       </c>
       <c r="AH70" t="n">
-        <v>87.23</v>
+        <v>73.02</v>
       </c>
       <c r="AI70" t="n">
         <v>1.0368</v>
@@ -9628,26 +9691,26 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>default-c454dca637a</t>
+          <t>default-d9e04639a2c</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>wqxhntH7cVkHGBGQHdmwHvGQQ8QOhy</t>
+          <t>zNojkfDZoro1z7t7fMQtUDJKvZGT6s</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 50000000, "_seconds": 1781339591}</t>
+          <t>{"_nanoseconds": 852000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1781339591050</v>
+        <v>1781339591852</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -9655,42 +9718,25 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="P71" t="n">
-        <v>1</v>
+        <v>0.45</v>
       </c>
       <c r="Q71" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="S71" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="U71" t="n">
-        <v>80</v>
-      </c>
-      <c r="V71" t="n">
-        <v>80</v>
+        <v>5.1</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>Base (Munich)</t>
+          <t>Base (Vienna)</t>
         </is>
       </c>
       <c r="X71" t="b">
         <v>0</v>
       </c>
-      <c r="Y71" t="inlineStr"/>
       <c r="Z71" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="AC71" t="n">
-        <v>4.6</v>
+        <v>2.85</v>
       </c>
       <c r="AD71" t="inlineStr">
         <is>
-          <t>Swaen Munich Light</t>
+          <t>Swaen Vienna</t>
         </is>
       </c>
       <c r="AE71" t="b">
@@ -9703,16 +9749,13 @@
         </is>
       </c>
       <c r="AH71" t="n">
-        <v>10.9</v>
+        <v>14.29</v>
       </c>
       <c r="AI71" t="n">
-        <v>1.035</v>
+        <v>1.03588</v>
       </c>
       <c r="AJ71" t="n">
-        <v>75.37</v>
-      </c>
-      <c r="AK71" t="n">
-        <v>11.7</v>
+        <v>78</v>
       </c>
       <c r="AL71" t="inlineStr"/>
       <c r="AM71" t="inlineStr">
@@ -9750,26 +9793,26 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>default-25ba5c7007d</t>
+          <t>default-c454dca637a</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>lBdAIVmlcp7FjYPSV55HleXloB6alW</t>
+          <t>wqxhntH7cVkHGBGQHdmwHvGQQ8QOhy</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 491000000, "_seconds": 1781339589}</t>
+          <t>{"_nanoseconds": 50000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I72" t="n">
-        <v>1781339589491</v>
+        <v>1781339591050</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -9777,48 +9820,64 @@
         </is>
       </c>
       <c r="L72" t="n">
-        <v>0.06</v>
+        <v>0.35</v>
+      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="P72" t="n">
+        <v>1</v>
       </c>
       <c r="Q72" t="n">
-        <v>61</v>
+        <v>6.6</v>
+      </c>
+      <c r="S72" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="U72" t="n">
+        <v>80</v>
+      </c>
+      <c r="V72" t="n">
+        <v>80</v>
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>Crystal/Caramel</t>
+          <t>Base (Munich)</t>
         </is>
       </c>
       <c r="X72" t="b">
         <v>0</v>
       </c>
+      <c r="Y72" t="inlineStr"/>
       <c r="Z72" t="n">
-        <v>1.36</v>
+        <v>2.54</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>4.6</v>
       </c>
       <c r="AD72" t="inlineStr">
         <is>
-          <t>GoldSwaen Classic</t>
+          <t>Swaen Munich Light</t>
         </is>
       </c>
       <c r="AE72" t="b">
         <v>0</v>
       </c>
-      <c r="AF72" t="inlineStr">
-        <is>
-          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
-        </is>
-      </c>
+      <c r="AF72" t="inlineStr"/>
       <c r="AG72" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
       <c r="AH72" t="n">
-        <v>1.87</v>
+        <v>11.11</v>
       </c>
       <c r="AI72" t="n">
-        <v>1.034</v>
+        <v>1.035</v>
       </c>
       <c r="AJ72" t="n">
-        <v>73.9130435</v>
+        <v>75.37</v>
+      </c>
+      <c r="AK72" t="n">
+        <v>11.7</v>
       </c>
       <c r="AL72" t="inlineStr"/>
       <c r="AM72" t="inlineStr">
@@ -9841,12 +9900,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
+          <t>yiPSN3Y6mmATMzlZ26e4uWlmbGRxaD</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>First lager</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -9854,52 +9913,54 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>default-HM41QfsZjsnkL2GS5s3sTYkVX5OKSM</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="n">
-        <v>0</v>
+          <t>default-25ba5c7007d</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>lBdAIVmlcp7FjYPSV55HleXloB6alW</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 491000000, "_seconds": 1781339589}</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>1781339589491</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
       </c>
       <c r="L73" t="n">
-        <v>3</v>
-      </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="P73" t="n">
-        <v>1.5</v>
+        <v>0.05</v>
       </c>
       <c r="Q73" t="n">
-        <v>1.8527919</v>
-      </c>
-      <c r="S73" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Crystal/Caramel</t>
         </is>
       </c>
       <c r="X73" t="b">
         <v>0</v>
       </c>
-      <c r="Y73" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB73" t="n">
-        <v>100</v>
-      </c>
-      <c r="AC73" t="n">
-        <v>4.5</v>
+      <c r="Z73" t="n">
+        <v>1.36</v>
       </c>
       <c r="AD73" t="inlineStr">
         <is>
-          <t>Clear Choice Malt ® Extra Pale</t>
+          <t>GoldSwaen Classic</t>
         </is>
       </c>
       <c r="AE73" t="b">
@@ -9907,30 +9968,27 @@
       </c>
       <c r="AF73" t="inlineStr">
         <is>
-          <t>Clear Choice Malt ® does not contain polyphenols thus reducing the risk of haze formation, increasing shelf life and reducing cold conditioning costs</t>
+          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
         </is>
       </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="AH73" t="n">
-        <v>68.18000000000001</v>
+        <v>1.59</v>
       </c>
       <c r="AI73" t="n">
-        <v>1.038</v>
+        <v>1.034</v>
       </c>
       <c r="AJ73" t="n">
-        <v>81.5</v>
-      </c>
-      <c r="AK73" t="n">
-        <v>10.1</v>
+        <v>73.9130435</v>
       </c>
       <c r="AL73" t="inlineStr"/>
       <c r="AM73" t="inlineStr">
         <is>
-          <t>Crisp</t>
+          <t>The Swaen</t>
         </is>
       </c>
       <c r="AN73" t="inlineStr">
@@ -9964,7 +10022,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>default-x1sQkldAFEgNTfYCHtBq70SjihT1F8</t>
+          <t>default-HM41QfsZjsnkL2GS5s3sTYkVX5OKSM</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
@@ -9975,21 +10033,21 @@
         <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M74" t="inlineStr"/>
       <c r="P74" t="n">
         <v>1.5</v>
       </c>
       <c r="Q74" t="n">
-        <v>3.9593909</v>
+        <v>1.8527919</v>
       </c>
       <c r="S74" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>Base (Vienna)</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="X74" t="b">
@@ -10006,7 +10064,7 @@
       </c>
       <c r="AD74" t="inlineStr">
         <is>
-          <t>Vienna Malt</t>
+          <t>Clear Choice Malt ® Extra Pale</t>
         </is>
       </c>
       <c r="AE74" t="b">
@@ -10014,7 +10072,7 @@
       </c>
       <c r="AF74" t="inlineStr">
         <is>
-          <t>Vienna malt is produced on a conventional kiln and provides a light golden hue</t>
+          <t>Clear Choice Malt ® does not contain polyphenols thus reducing the risk of haze formation, increasing shelf life and reducing cold conditioning costs</t>
         </is>
       </c>
       <c r="AG74" t="inlineStr">
@@ -10023,16 +10081,16 @@
         </is>
       </c>
       <c r="AH74" t="n">
-        <v>22.73</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="AI74" t="n">
-        <v>1.037</v>
+        <v>1.038</v>
       </c>
       <c r="AJ74" t="n">
-        <v>80</v>
+        <v>81.5</v>
       </c>
       <c r="AK74" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="AL74" t="inlineStr"/>
       <c r="AM74" t="inlineStr">
@@ -10068,75 +10126,83 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>default-sabmjufsad</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>TbX832JbWp5BHVi5ATe4AaXk3nMfr9</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
-        </is>
-      </c>
-      <c r="I75" t="n">
-        <v>1706434202728</v>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>2.10.5</t>
-        </is>
+          <t>default-x1sQkldAFEgNTfYCHtBq70SjihT1F8</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="n">
+        <v>0</v>
       </c>
       <c r="L75" t="n">
-        <v>0.3</v>
+        <v>1</v>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="P75" t="n">
+        <v>1.5</v>
       </c>
       <c r="Q75" t="n">
-        <v>2</v>
+        <v>3.9593909</v>
+      </c>
+      <c r="S75" t="n">
+        <v>50</v>
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Base (Vienna)</t>
         </is>
       </c>
       <c r="X75" t="b">
         <v>0</v>
       </c>
-      <c r="Z75" t="n">
-        <v>-2.29</v>
+      <c r="Y75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>4.5</v>
       </c>
       <c r="AD75" t="inlineStr">
         <is>
-          <t>Pale Malt 2-Row</t>
+          <t>Vienna Malt</t>
         </is>
       </c>
       <c r="AE75" t="b">
         <v>0</v>
       </c>
-      <c r="AF75" t="inlineStr"/>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>Vienna malt is produced on a conventional kiln and provides a light golden hue</t>
+        </is>
+      </c>
       <c r="AG75" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="AH75" t="n">
-        <v>6.82</v>
+        <v>22.73</v>
       </c>
       <c r="AI75" t="n">
-        <v>1.036</v>
+        <v>1.037</v>
+      </c>
+      <c r="AJ75" t="n">
+        <v>80</v>
+      </c>
+      <c r="AK75" t="n">
+        <v>9.6</v>
       </c>
       <c r="AL75" t="inlineStr"/>
       <c r="AM75" t="inlineStr">
         <is>
-          <t>SAB</t>
+          <t>Crisp</t>
         </is>
       </c>
       <c r="AN75" t="inlineStr">
@@ -10147,9 +10213,7 @@
       <c r="AO75" t="inlineStr"/>
       <c r="AP75" t="inlineStr"/>
       <c r="AQ75" t="inlineStr"/>
-      <c r="AR75" t="b">
-        <v>0</v>
-      </c>
+      <c r="AR75" t="inlineStr"/>
       <c r="AS75" t="inlineStr"/>
       <c r="AT75" t="inlineStr"/>
     </row>
@@ -10171,108 +10235,73 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 526000000, "_seconds": 1706434203}</t>
+          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>default-4c1345c</t>
+          <t>default-sabmjufsad</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KAv9WQAuhq3uEgowTzBf8YrHtXE4LO</t>
+          <t>TbX832JbWp5BHVi5ATe4AaXk3nMfr9</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 140000000, "_seconds": 1712314604}</t>
+          <t>{"_nanoseconds": 728000000, "_seconds": 1706434202}</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>1712314604140</v>
+        <v>1706434202728</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2.10.6</t>
-        </is>
-      </c>
-      <c r="K76" t="n">
+          <t>2.10.5</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q76" t="n">
         <v>2</v>
       </c>
-      <c r="L76" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M76" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="P76" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Q76" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="S76" t="n">
-        <v>0</v>
-      </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>Acidulated</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="X76" t="b">
         <v>0</v>
       </c>
-      <c r="Y76" t="n">
-        <v>0</v>
-      </c>
       <c r="Z76" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="AB76" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC76" t="n">
-        <v>4</v>
+        <v>-2.29</v>
       </c>
       <c r="AD76" t="inlineStr">
         <is>
-          <t>Acidulated</t>
+          <t>Pale Malt 2-Row</t>
         </is>
       </c>
       <c r="AE76" t="b">
         <v>0</v>
       </c>
-      <c r="AF76" t="inlineStr">
-        <is>
-          <t>Used in Germany to lower PH levels without resorting to chemicals. Lowers mash pH levels, lightens color, improves flavor stability.</t>
-        </is>
-      </c>
+      <c r="AF76" t="inlineStr"/>
       <c r="AG76" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="AH76" t="n">
-        <v>2.27</v>
+        <v>6.82</v>
       </c>
       <c r="AI76" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AJ76" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="AK76" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL76" t="inlineStr">
-        <is>
-          <t>Pale Liquid Extract</t>
-        </is>
-      </c>
+        <v>1.036</v>
+      </c>
+      <c r="AL76" t="inlineStr"/>
       <c r="AM76" t="inlineStr">
         <is>
-          <t>Weyermann</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="AN76" t="inlineStr">
@@ -10283,19 +10312,21 @@
       <c r="AO76" t="inlineStr"/>
       <c r="AP76" t="inlineStr"/>
       <c r="AQ76" t="inlineStr"/>
-      <c r="AR76" t="inlineStr"/>
+      <c r="AR76" t="b">
+        <v>0</v>
+      </c>
       <c r="AS76" t="inlineStr"/>
       <c r="AT76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
+          <t>zLftyphr8T4DoHNZs92dj1mO4gPXZq</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Smash - Citra</t>
+          <t>First lager</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -10303,69 +10334,110 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 526000000, "_seconds": 1706434203}</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>new-eNDTHs2wb879roS3Dq1orvcb3ATgbD</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+          <t>default-4c1345c</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>KAv9WQAuhq3uEgowTzBf8YrHtXE4LO</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 140000000, "_seconds": 1712314604}</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>1712314604140</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>2</v>
+      </c>
       <c r="L77" t="n">
-        <v>13.18</v>
-      </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
+        <v>0.1</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="P77" t="n">
+        <v>1.5</v>
+      </c>
       <c r="Q77" t="n">
-        <v>3</v>
-      </c>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
-      <c r="T77" t="inlineStr"/>
-      <c r="U77" t="inlineStr"/>
-      <c r="V77" t="inlineStr"/>
+        <v>1.8</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>Base (Maris Otter)</t>
-        </is>
-      </c>
-      <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
-      <c r="Z77" t="inlineStr"/>
-      <c r="AA77" t="inlineStr"/>
-      <c r="AB77" t="inlineStr"/>
-      <c r="AC77" t="inlineStr"/>
+          <t>Acidulated</t>
+        </is>
+      </c>
+      <c r="X77" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="AB77" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>4</v>
+      </c>
       <c r="AD77" t="inlineStr">
         <is>
-          <t>Pale Malt, Maris Otter</t>
-        </is>
-      </c>
-      <c r="AE77" t="inlineStr"/>
-      <c r="AF77" t="inlineStr"/>
+          <t>Acidulated</t>
+        </is>
+      </c>
+      <c r="AE77" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF77" t="inlineStr">
+        <is>
+          <t>Used in Germany to lower PH levels without resorting to chemicals. Lowers mash pH levels, lightens color, improves flavor stability.</t>
+        </is>
+      </c>
       <c r="AG77" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="AH77" t="n">
-        <v>100</v>
+        <v>2.27</v>
       </c>
       <c r="AI77" t="n">
-        <v>1.03795</v>
+        <v>1.03</v>
       </c>
       <c r="AJ77" t="n">
-        <v>82.5</v>
-      </c>
-      <c r="AK77" t="inlineStr"/>
-      <c r="AL77" t="inlineStr"/>
+        <v>65.2</v>
+      </c>
+      <c r="AK77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL77" t="inlineStr">
+        <is>
+          <t>Pale Liquid Extract</t>
+        </is>
+      </c>
       <c r="AM77" t="inlineStr">
         <is>
-          <t>Maris Otter</t>
+          <t>Weyermann</t>
         </is>
       </c>
       <c r="AN77" t="inlineStr">
@@ -10378,21 +10450,17 @@
       <c r="AQ77" t="inlineStr"/>
       <c r="AR77" t="inlineStr"/>
       <c r="AS77" t="inlineStr"/>
-      <c r="AT77" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
+      <c r="AT77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
+          <t>ldKgMhTaCxdOMCepRg4HaR2lskjbXE</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Saison</t>
+          <t>Smash - Citra</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -10400,78 +10468,69 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>default-c3ff8bb88f9</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>tqtVycoLMiKmJMplyu7GCIAsAeeETL</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>{"_nanoseconds": 476000000, "_seconds": 1781339591}</t>
-        </is>
-      </c>
-      <c r="I78" t="n">
-        <v>1781339591476</v>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>3.0.1</t>
-        </is>
-      </c>
+          <t>new-eNDTHs2wb879roS3Dq1orvcb3ATgbD</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
       <c r="L78" t="n">
-        <v>2.4</v>
-      </c>
+        <v>13.18</v>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
       <c r="Q78" t="n">
-        <v>1.9</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="inlineStr"/>
       <c r="W78" t="inlineStr">
         <is>
-          <t>Base (Pilsner)</t>
-        </is>
-      </c>
-      <c r="X78" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z78" t="n">
-        <v>6.7</v>
-      </c>
+          <t>Base (Maris Otter)</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr">
         <is>
-          <t>Swaen Pilsner</t>
-        </is>
-      </c>
-      <c r="AE78" t="b">
-        <v>0</v>
-      </c>
+          <t>Pale Malt, Maris Otter</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr"/>
       <c r="AF78" t="inlineStr"/>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="AH78" t="n">
-        <v>78.43000000000001</v>
+        <v>100</v>
       </c>
       <c r="AI78" t="n">
-        <v>1.0368</v>
+        <v>1.03795</v>
       </c>
       <c r="AJ78" t="n">
-        <v>80</v>
-      </c>
+        <v>82.5</v>
+      </c>
+      <c r="AK78" t="inlineStr"/>
       <c r="AL78" t="inlineStr"/>
       <c r="AM78" t="inlineStr">
         <is>
-          <t>The Swaen</t>
+          <t>Maris Otter</t>
         </is>
       </c>
       <c r="AN78" t="inlineStr">
@@ -10484,7 +10543,11 @@
       <c r="AQ78" t="inlineStr"/>
       <c r="AR78" t="inlineStr"/>
       <c r="AS78" t="inlineStr"/>
-      <c r="AT78" t="inlineStr"/>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10504,26 +10567,26 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>default-d9e04639a2c</t>
+          <t>default-c3ff8bb88f9</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>zNojkfDZoro1z7t7fMQtUDJKvZGT6s</t>
+          <t>tqtVycoLMiKmJMplyu7GCIAsAeeETL</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 852000000, "_seconds": 1781339591}</t>
+          <t>{"_nanoseconds": 476000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>1781339591852</v>
+        <v>1781339591476</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -10531,25 +10594,25 @@
         </is>
       </c>
       <c r="L79" t="n">
-        <v>0.34</v>
+        <v>2.4</v>
       </c>
       <c r="Q79" t="n">
-        <v>5.1</v>
+        <v>1.9</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>Base (Vienna)</t>
+          <t>Base (Pilsner)</t>
         </is>
       </c>
       <c r="X79" t="b">
         <v>0</v>
       </c>
       <c r="Z79" t="n">
-        <v>2.85</v>
+        <v>6.7</v>
       </c>
       <c r="AD79" t="inlineStr">
         <is>
-          <t>Swaen Vienna</t>
+          <t>Swaen Pilsner</t>
         </is>
       </c>
       <c r="AE79" t="b">
@@ -10562,13 +10625,13 @@
         </is>
       </c>
       <c r="AH79" t="n">
-        <v>11.11</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="AI79" t="n">
-        <v>1.03588</v>
+        <v>1.0368</v>
       </c>
       <c r="AJ79" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AL79" t="inlineStr"/>
       <c r="AM79" t="inlineStr">
@@ -10606,71 +10669,81 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 526000000, "_seconds": 1719746358}</t>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>default-132c22b</t>
+          <t>default-d9e04639a2c</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>feD3na0a4sxySPUBRKwyBrSewo4G5I</t>
+          <t>zNojkfDZoro1z7t7fMQtUDJKvZGT6s</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 383000000, "_seconds": 1772634460}</t>
+          <t>{"_nanoseconds": 852000000, "_seconds": 1781339591}</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>1772634460383</v>
+        <v>1781339591852</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2.20.2</t>
+          <t>3.0.1</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="M80" t="n">
-        <v>1.22</v>
+        <v>0.34</v>
       </c>
       <c r="Q80" t="n">
-        <v>1</v>
+        <v>5.1</v>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Base (Vienna)</t>
+        </is>
       </c>
       <c r="X80" t="b">
         <v>0</v>
       </c>
       <c r="Z80" t="n">
-        <v>0</v>
+        <v>2.85</v>
       </c>
       <c r="AD80" t="inlineStr">
         <is>
-          <t>Sugar, Table (Sucrose)</t>
+          <t>Swaen Vienna</t>
         </is>
       </c>
       <c r="AE80" t="b">
         <v>0</v>
       </c>
       <c r="AF80" t="inlineStr"/>
-      <c r="AG80" t="inlineStr"/>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
       <c r="AH80" t="n">
-        <v>6.86</v>
+        <v>11.11</v>
       </c>
       <c r="AI80" t="n">
-        <v>1.046</v>
+        <v>1.03588</v>
       </c>
       <c r="AJ80" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="AL80" t="inlineStr"/>
-      <c r="AM80" t="inlineStr"/>
+      <c r="AM80" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
       <c r="AN80" t="inlineStr">
         <is>
-          <t>Sugar</t>
+          <t>Grain</t>
         </is>
       </c>
       <c r="AO80" t="inlineStr"/>
@@ -10698,101 +10771,71 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
+          <t>{"_nanoseconds": 526000000, "_seconds": 1719746358}</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>default-c454dca637a</t>
+          <t>default-132c22b</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>yKptvZxfGwlhwsenw2CQpv3yu9A5Qm</t>
+          <t>feD3na0a4sxySPUBRKwyBrSewo4G5I</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 905000000, "_seconds": 1785061180}</t>
+          <t>{"_nanoseconds": 383000000, "_seconds": 1772634460}</t>
         </is>
       </c>
       <c r="I81" t="n">
-        <v>1785061180905</v>
+        <v>1772634460383</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>3.0.1</t>
+          <t>2.20.2</t>
         </is>
       </c>
       <c r="L81" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="P81" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="M81" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="Q81" t="n">
         <v>1</v>
       </c>
-      <c r="Q81" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="S81" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="U81" t="n">
-        <v>80</v>
-      </c>
-      <c r="V81" t="n">
-        <v>80</v>
-      </c>
-      <c r="W81" t="inlineStr">
-        <is>
-          <t>Base (Munich)</t>
-        </is>
-      </c>
       <c r="X81" t="b">
         <v>0</v>
       </c>
-      <c r="Y81" t="inlineStr"/>
       <c r="Z81" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="AC81" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="AD81" t="inlineStr">
         <is>
-          <t>Swaen Munich Light</t>
+          <t>Sugar, Table (Sucrose)</t>
         </is>
       </c>
       <c r="AE81" t="b">
         <v>0</v>
       </c>
       <c r="AF81" t="inlineStr"/>
-      <c r="AG81" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
+      <c r="AG81" t="inlineStr"/>
       <c r="AH81" t="n">
-        <v>3.59</v>
+        <v>6.86</v>
       </c>
       <c r="AI81" t="n">
-        <v>1.035</v>
+        <v>1.046</v>
       </c>
       <c r="AJ81" t="n">
-        <v>75.37</v>
-      </c>
-      <c r="AK81" t="n">
-        <v>11.7</v>
+        <v>100</v>
       </c>
       <c r="AL81" t="inlineStr"/>
-      <c r="AM81" t="inlineStr">
-        <is>
-          <t>The Swaen</t>
-        </is>
-      </c>
+      <c r="AM81" t="inlineStr"/>
       <c r="AN81" t="inlineStr">
         <is>
-          <t>Grain</t>
+          <t>Sugar</t>
         </is>
       </c>
       <c r="AO81" t="inlineStr"/>
@@ -10805,12 +10848,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
+          <t>6uXxDtvdy8UOY2sOfjUUUeSVldFbeu</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Smash Mosaic</t>
+          <t>Saison</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -10820,26 +10863,26 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>default-c3ff8bb88f9</t>
+          <t>default-c454dca637a</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>BglUUy5uFFFvFjGd9EbIYIPvAJyyIE</t>
+          <t>yKptvZxfGwlhwsenw2CQpv3yu9A5Qm</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 508000000, "_seconds": 1785061181}</t>
+          <t>{"_nanoseconds": 905000000, "_seconds": 1785061180}</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>1785061181508</v>
+        <v>1785061180905</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -10847,25 +10890,42 @@
         </is>
       </c>
       <c r="L82" t="n">
-        <v>3</v>
+        <v>0.11</v>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="P82" t="n">
+        <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>1.9</v>
+        <v>6.6</v>
+      </c>
+      <c r="S82" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="U82" t="n">
+        <v>80</v>
+      </c>
+      <c r="V82" t="n">
+        <v>80</v>
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>Base (Pilsner)</t>
+          <t>Base (Munich)</t>
         </is>
       </c>
       <c r="X82" t="b">
         <v>0</v>
       </c>
+      <c r="Y82" t="inlineStr"/>
       <c r="Z82" t="n">
-        <v>4.4</v>
+        <v>2.19</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>4.6</v>
       </c>
       <c r="AD82" t="inlineStr">
         <is>
-          <t>Swaen Pilsner</t>
+          <t>Swaen Munich Light</t>
         </is>
       </c>
       <c r="AE82" t="b">
@@ -10878,13 +10938,16 @@
         </is>
       </c>
       <c r="AH82" t="n">
-        <v>100</v>
+        <v>3.59</v>
       </c>
       <c r="AI82" t="n">
-        <v>1.0368</v>
+        <v>1.035</v>
       </c>
       <c r="AJ82" t="n">
-        <v>80</v>
+        <v>75.37</v>
+      </c>
+      <c r="AK82" t="n">
+        <v>11.7</v>
       </c>
       <c r="AL82" t="inlineStr"/>
       <c r="AM82" t="inlineStr">
@@ -10907,12 +10970,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
+          <t>rJhcyGonoBkZSA8onOHB3KYOWjvOFo</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Smash shoddy</t>
+          <t>Smash Mosaic</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -11009,12 +11072,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TtkyFZuS1krih6K7d2BW7nY3qFmYPZ</t>
+          <t>dXad4F2tnZ5bYPr0H7o1LxG5LkDq1C</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Kalahari blond 16 liter</t>
+          <t>Smash shoddy</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -11034,16 +11097,16 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>GOG6rzO2xrYYSto1fMsaU5lUVzV9v7</t>
+          <t>BglUUy5uFFFvFjGd9EbIYIPvAJyyIE</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 7000000, "_seconds": 1786789728}</t>
+          <t>{"_nanoseconds": 508000000, "_seconds": 1785061181}</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>1786789728007</v>
+        <v>1785061181508</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -11051,7 +11114,7 @@
         </is>
       </c>
       <c r="L84" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="Q84" t="n">
         <v>1.9</v>
@@ -11065,7 +11128,7 @@
         <v>0</v>
       </c>
       <c r="Z84" t="n">
-        <v>11.4</v>
+        <v>4.4</v>
       </c>
       <c r="AD84" t="inlineStr">
         <is>
@@ -11082,7 +11145,7 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>77.5</v>
+        <v>100</v>
       </c>
       <c r="AI84" t="n">
         <v>1.0368</v>
@@ -11126,26 +11189,26 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 983000000, "_seconds": 1775498604}</t>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>default-d9e04639a2c</t>
+          <t>default-c3ff8bb88f9</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>vNwfSmBlJ1e4z5jdNJOlLtSxOILZid</t>
+          <t>GOG6rzO2xrYYSto1fMsaU5lUVzV9v7</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>{"_nanoseconds": 15000000, "_seconds": 1785061182}</t>
+          <t>{"_nanoseconds": 7000000, "_seconds": 1786789728}</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>1785061182015</v>
+        <v>1786789728007</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -11153,25 +11216,25 @@
         </is>
       </c>
       <c r="L85" t="n">
-        <v>0.64</v>
+        <v>3.3</v>
       </c>
       <c r="Q85" t="n">
-        <v>5.1</v>
+        <v>1.9</v>
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>Base (Vienna)</t>
+          <t>Base (Pilsner)</t>
         </is>
       </c>
       <c r="X85" t="b">
         <v>0</v>
       </c>
       <c r="Z85" t="n">
-        <v>2.4</v>
+        <v>11.4</v>
       </c>
       <c r="AD85" t="inlineStr">
         <is>
-          <t>Swaen Vienna</t>
+          <t>Swaen Pilsner</t>
         </is>
       </c>
       <c r="AE85" t="b">
@@ -11184,13 +11247,13 @@
         </is>
       </c>
       <c r="AH85" t="n">
-        <v>16</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="AI85" t="n">
-        <v>1.03588</v>
+        <v>1.0368</v>
       </c>
       <c r="AJ85" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AL85" t="inlineStr"/>
       <c r="AM85" t="inlineStr">
@@ -11226,83 +11289,98 @@
           <t>Fermentable</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 835000000, "_seconds": 1775498551}</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>default-MSMYXD2BJLGqRAHlZVbqdHLIa0VzoF</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="n">
-        <v>0</v>
+          <t>default-c454dca637a</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>8RBzx8WZSkSmbLLiWSJhSrf0Ak2Trz</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 681000000, "_seconds": 1788086444}</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>1788086444681</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
       </c>
       <c r="L86" t="n">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="P86" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>2.5380711</v>
+        <v>6.6</v>
       </c>
       <c r="S86" t="n">
-        <v>0</v>
+        <v>18.2</v>
+      </c>
+      <c r="U86" t="n">
+        <v>80</v>
+      </c>
+      <c r="V86" t="n">
+        <v>80</v>
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>Base (Wheat)</t>
+          <t>Base (Munich)</t>
         </is>
       </c>
       <c r="X86" t="b">
         <v>0</v>
       </c>
-      <c r="Y86" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB86" t="n">
-        <v>25</v>
+      <c r="Y86" t="inlineStr"/>
+      <c r="Z86" t="n">
+        <v>2.04</v>
       </c>
       <c r="AC86" t="n">
-        <v>10</v>
+        <v>4.6</v>
       </c>
       <c r="AD86" t="inlineStr">
         <is>
-          <t>Torrefied Wheat</t>
+          <t>Swaen Munich Light</t>
         </is>
       </c>
       <c r="AE86" t="b">
         <v>0</v>
       </c>
-      <c r="AF86" t="inlineStr">
-        <is>
-          <t>Pre-cooked, non-malted cereals provide the brewer with the opportunity for product differentiation. Flaked products can be added directly to the mash without the need for milling.</t>
-        </is>
-      </c>
+      <c r="AF86" t="inlineStr"/>
       <c r="AG86" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>6.5</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="AI86" t="n">
-        <v>1.038</v>
+        <v>1.035</v>
       </c>
       <c r="AJ86" t="n">
-        <v>82</v>
+        <v>75.37</v>
       </c>
       <c r="AK86" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
       <c r="AL86" t="inlineStr"/>
       <c r="AM86" t="inlineStr">
         <is>
-          <t>Crisp</t>
+          <t>The Swaen</t>
         </is>
       </c>
       <c r="AN86" t="inlineStr">
@@ -11317,8 +11395,811 @@
       <c r="AS86" t="inlineStr"/>
       <c r="AT86" t="inlineStr"/>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TtkyFZuS1krih6K7d2BW7nY3qFmYPZ</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Kalahari blond 16 liter</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>default-MSMYXD2BJLGqRAHlZVbqdHLIa0VzoF</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="P87" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>2.5380711</v>
+      </c>
+      <c r="S87" t="n">
+        <v>0</v>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>Base (Wheat)</t>
+        </is>
+      </c>
+      <c r="X87" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>Torrefied Wheat</t>
+        </is>
+      </c>
+      <c r="AE87" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>Pre-cooked, non-malted cereals provide the brewer with the opportunity for product differentiation. Flaked products can be added directly to the mash without the need for milling.</t>
+        </is>
+      </c>
+      <c r="AG87" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH87" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="AI87" t="n">
+        <v>1.038</v>
+      </c>
+      <c r="AJ87" t="n">
+        <v>82</v>
+      </c>
+      <c r="AK87" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL87" t="inlineStr"/>
+      <c r="AM87" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN87" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO87" t="inlineStr"/>
+      <c r="AP87" t="inlineStr"/>
+      <c r="AQ87" t="inlineStr"/>
+      <c r="AR87" t="inlineStr"/>
+      <c r="AS87" t="inlineStr"/>
+      <c r="AT87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 499000000, "_seconds": 1706434201}</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>default-e6ba5b8</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>OTZvOBRODuXjmguhpWZUQ4uz2r8zid</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 714000000, "_seconds": 1721546982}</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>1721546982714</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="P88" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>3.2994924</v>
+      </c>
+      <c r="S88" t="n">
+        <v>53</v>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Base (Maris Otter)</t>
+        </is>
+      </c>
+      <c r="X88" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>-4.59</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>Finest Maris Otter® Ale Malt</t>
+        </is>
+      </c>
+      <c r="AE88" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>The consistently reliable Maris Otter® continues to provide the qualities expected by the brewer</t>
+        </is>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH88" t="n">
+        <v>75</v>
+      </c>
+      <c r="AI88" t="n">
+        <v>1.038</v>
+      </c>
+      <c r="AJ88" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="AK88" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL88" t="inlineStr"/>
+      <c r="AM88" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN88" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO88" t="inlineStr"/>
+      <c r="AP88" t="inlineStr"/>
+      <c r="AQ88" t="inlineStr"/>
+      <c r="AR88" t="inlineStr"/>
+      <c r="AS88" t="inlineStr"/>
+      <c r="AT88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 14000000, "_seconds": 1787844774}</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>default-MSMYXD2BJLGqRAHlZVbqdHLIa0VzoF</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>RfTzDOwr83mMgEx7DXAJqSmiTnkaet</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 14000000, "_seconds": 1787844774}</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>1787844774014</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="P89" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>2.5380711</v>
+      </c>
+      <c r="S89" t="n">
+        <v>0</v>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>Base (Wheat)</t>
+        </is>
+      </c>
+      <c r="X89" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB89" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>Torrefied Wheat</t>
+        </is>
+      </c>
+      <c r="AE89" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
+          <t>Pre-cooked, non-malted cereals provide the brewer with the opportunity for product differentiation. Flaked products can be added directly to the mash without the need for milling.</t>
+        </is>
+      </c>
+      <c r="AG89" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH89" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AI89" t="n">
+        <v>1.038</v>
+      </c>
+      <c r="AJ89" t="n">
+        <v>82</v>
+      </c>
+      <c r="AK89" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL89" t="inlineStr"/>
+      <c r="AM89" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN89" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO89" t="inlineStr"/>
+      <c r="AP89" t="inlineStr"/>
+      <c r="AQ89" t="inlineStr"/>
+      <c r="AR89" t="inlineStr"/>
+      <c r="AS89" t="inlineStr"/>
+      <c r="AT89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 306000000, "_seconds": 1776345994}</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>default-25ba5c7007d</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>1J9fe3tUex3oOKOPk0F51aZTCC6NvP</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 983000000, "_seconds": 1785061179}</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>1785061179983</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>61</v>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>Crystal/Caramel</t>
+        </is>
+      </c>
+      <c r="X90" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>GoldSwaen Classic</t>
+        </is>
+      </c>
+      <c r="AE90" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>5-10% for dark beers, 1-5% for light beer, Pale Ale 20%</t>
+        </is>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH90" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="AI90" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="AJ90" t="n">
+        <v>73.9130435</v>
+      </c>
+      <c r="AL90" t="inlineStr"/>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN90" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO90" t="inlineStr"/>
+      <c r="AP90" t="inlineStr"/>
+      <c r="AQ90" t="inlineStr"/>
+      <c r="AR90" t="inlineStr"/>
+      <c r="AS90" t="inlineStr"/>
+      <c r="AT90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 593000000, "_seconds": 1776345977}</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>default-29dda1b5335</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>R3yyMXfk1baparTfJ2ej9HajPEgito</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 919000000, "_seconds": 1781339588}</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>1781339588919</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>329.949239</v>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>Crystal/Caramel</t>
+        </is>
+      </c>
+      <c r="X91" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>BlackSwaen Coffee</t>
+        </is>
+      </c>
+      <c r="AE91" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF91" t="inlineStr"/>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH91" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="AI91" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>60.8695652</v>
+      </c>
+      <c r="AL91" t="inlineStr"/>
+      <c r="AM91" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN91" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO91" t="inlineStr"/>
+      <c r="AP91" t="inlineStr"/>
+      <c r="AQ91" t="n">
+        <v>244.1</v>
+      </c>
+      <c r="AR91" t="inlineStr"/>
+      <c r="AS91" t="inlineStr"/>
+      <c r="AT91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 563000000, "_seconds": 1775498626}</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>default-c3ff8bb88f9</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Ou91CMOYwCNfTOIWjNXLjhWUBAxN7m</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 244000000, "_seconds": 1788086445}</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>1788086445244</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Base (Pilsner)</t>
+        </is>
+      </c>
+      <c r="X92" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>Swaen Pilsner</t>
+        </is>
+      </c>
+      <c r="AE92" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF92" t="inlineStr"/>
+      <c r="AG92" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="AH92" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="AI92" t="n">
+        <v>1.0368</v>
+      </c>
+      <c r="AJ92" t="n">
+        <v>80</v>
+      </c>
+      <c r="AL92" t="inlineStr"/>
+      <c r="AM92" t="inlineStr">
+        <is>
+          <t>The Swaen</t>
+        </is>
+      </c>
+      <c r="AN92" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO92" t="inlineStr"/>
+      <c r="AP92" t="inlineStr"/>
+      <c r="AQ92" t="inlineStr"/>
+      <c r="AR92" t="inlineStr"/>
+      <c r="AS92" t="inlineStr"/>
+      <c r="AT92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Fermentable</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 212000000, "_seconds": 1775499019}</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>default-c5e48c4</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>9mGQgdZMjKAOZQSjsXo7x5DVWTbPaC</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 714000000, "_seconds": 1777108185}</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>1777108185714</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>3.0.0</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="P93" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>529.4416244</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0</v>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Roasted</t>
+        </is>
+      </c>
+      <c r="X93" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB93" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>Chocolate Malt</t>
+        </is>
+      </c>
+      <c r="AE93" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF93" t="inlineStr">
+        <is>
+          <t>Gives dry, toasty flavours to rich, dark beers</t>
+        </is>
+      </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="AH93" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AI93" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="AJ93" t="n">
+        <v>72</v>
+      </c>
+      <c r="AK93" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL93" t="inlineStr"/>
+      <c r="AM93" t="inlineStr">
+        <is>
+          <t>Crisp</t>
+        </is>
+      </c>
+      <c r="AN93" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="AO93" t="inlineStr"/>
+      <c r="AP93" t="inlineStr"/>
+      <c r="AQ93" t="inlineStr"/>
+      <c r="AR93" t="inlineStr"/>
+      <c r="AS93" t="inlineStr"/>
+      <c r="AT93" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AT86"/>
+  <autoFilter ref="A1:AT93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11329,7 +12210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP79"/>
+  <dimension ref="A1:AP81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16640,7 +17521,7 @@
         <v>30</v>
       </c>
       <c r="Q53" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -16741,7 +17622,7 @@
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="Q54" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="T54" t="inlineStr">
         <is>
@@ -16811,11 +17692,11 @@
         <v>10</v>
       </c>
       <c r="H55" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="Q55" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -16885,11 +17766,11 @@
         <v>10</v>
       </c>
       <c r="H56" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="N56" t="inlineStr"/>
       <c r="Q56" t="n">
-        <v>8.800000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -16961,11 +17842,11 @@
         <v>5.5</v>
       </c>
       <c r="H57" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="Q57" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
@@ -19047,7 +19928,7 @@
         <v>30</v>
       </c>
       <c r="Q77" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -19317,8 +20198,230 @@
         <v>45</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>default-southernaroma</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>4</v>
+      </c>
+      <c r="H80" t="n">
+        <v>30</v>
+      </c>
+      <c r="J80" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="N80" t="b">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Southern Aroma</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Fields of flowers, Dried Herbs, Parsley, Grain, Straw, Sunny hayfield</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>Saaz, Hallertauer Mittelfrueh</t>
+        </is>
+      </c>
+      <c r="Z80" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr"/>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 473000000, "_seconds": 1719746363}</t>
+        </is>
+      </c>
+      <c r="AH80" t="inlineStr">
+        <is>
+          <t>XCWEvYDmMFt4NFK6nyts7Bg9HJD3vR</t>
+        </is>
+      </c>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 473000000, "_seconds": 1719746363}</t>
+        </is>
+      </c>
+      <c r="AJ80" t="n">
+        <v>1719746363473</v>
+      </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="AL80" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AM80" t="inlineStr"/>
+      <c r="AN80" t="inlineStr"/>
+      <c r="AO80" t="inlineStr"/>
+      <c r="AP80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Hop</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>default-southernaroma</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>4</v>
+      </c>
+      <c r="H81" t="n">
+        <v>20</v>
+      </c>
+      <c r="J81" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="N81" t="b">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Southern Aroma</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Fields of flowers, Dried Herbs, Parsley, Grain, Straw, Sunny hayfield</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>Saaz, Hallertauer Mittelfrueh</t>
+        </is>
+      </c>
+      <c r="Y81" t="n">
+        <v>80</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>Pellet</t>
+        </is>
+      </c>
+      <c r="AB81" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>Aroma</t>
+        </is>
+      </c>
+      <c r="AD81" t="inlineStr"/>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 473000000, "_seconds": 1719746363}</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>XCWEvYDmMFt4NFK6nyts7Bg9HJD3vR</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 473000000, "_seconds": 1719746363}</t>
+        </is>
+      </c>
+      <c r="AJ81" t="n">
+        <v>1719746363473</v>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="AL81" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AN81" t="inlineStr"/>
+      <c r="AO81" t="inlineStr"/>
+      <c r="AP81" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AP79"/>
+  <autoFilter ref="A1:AP81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19329,7 +20432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL25"/>
+  <dimension ref="A1:AL26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -22155,7 +23258,11 @@
           <t>pkg</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use 7 or 8 grams. </t>
+        </is>
+      </c>
       <c r="AA25" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
@@ -22169,8 +23276,112 @@
       <c r="AK25" t="inlineStr"/>
       <c r="AL25" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Yeast</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>default-Nus0U2QXJCoeFdPx6G7BNazD19W04F</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>85</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>A British-style ale yeast that is characterized by high attenuation, low ester formation during fermentation, and high ABV tolerance. A good top-fermenting yeast strain that is a great choice for pale ales, ambers, porters, and stouts.
+Oxygenation and/or rehydration for generation 0 may be beneficial, but not necessary.</t>
+        </is>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Dry</t>
+        </is>
+      </c>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>WHC Lab</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>14</v>
+      </c>
+      <c r="R26" t="n">
+        <v>85</v>
+      </c>
+      <c r="S26" t="n">
+        <v>22</v>
+      </c>
+      <c r="T26" t="n">
+        <v>78</v>
+      </c>
+      <c r="U26" t="n">
+        <v>18</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>WHC Old English</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Old English</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>Ale</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>pkg</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AL25"/>
+  <autoFilter ref="A1:AL26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22181,7 +23392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB140"/>
+  <dimension ref="A1:AB147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -33901,8 +35112,605 @@
       <c r="AA140" t="inlineStr"/>
       <c r="AB140" t="inlineStr"/>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 20000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>default-2302b0</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>dHzf3qHIzqCVtmbVlXqvCaYqHnAPxv</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 69000000, "_seconds": 1781339599}</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>1781339599069</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>2</v>
+      </c>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="b">
+        <v>0</v>
+      </c>
+      <c r="N141" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Baking Soda (NaHCO3)</t>
+        </is>
+      </c>
+      <c r="Q141" t="b">
+        <v>0</v>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U141" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y141" t="inlineStr"/>
+      <c r="Z141" t="inlineStr"/>
+      <c r="AA141" t="inlineStr"/>
+      <c r="AB141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 152000000, "_seconds": 1699176797}</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>default-3b1827</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>hVBLHIBRmfjgeCufI6dYL7ohKfkror</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 760000000, "_seconds": 1788086587}</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>1788086587760</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>2</v>
+      </c>
+      <c r="M142" t="b">
+        <v>0</v>
+      </c>
+      <c r="N142" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Calcium Chloride (CaCl2)</t>
+        </is>
+      </c>
+      <c r="Q142" t="b">
+        <v>0</v>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U142" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y142" t="inlineStr"/>
+      <c r="Z142" t="inlineStr"/>
+      <c r="AA142" t="inlineStr"/>
+      <c r="AB142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1699176796}</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>default-1f88df</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>hOo044cGVkLCieJyI8rCtsPKtcdSbS</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 254000000, "_seconds": 1788086560}</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>1788086560254</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>2</v>
+      </c>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="b">
+        <v>0</v>
+      </c>
+      <c r="N143" t="n">
+        <v>931.5</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Gypsum (CaSO4)</t>
+        </is>
+      </c>
+      <c r="Q143" t="b">
+        <v>0</v>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U143" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y143" t="inlineStr"/>
+      <c r="Z143" t="inlineStr"/>
+      <c r="AA143" t="inlineStr"/>
+      <c r="AB143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 828000000, "_seconds": 1706434207}</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>default-07adb1</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>T70jwvYnCpjZXjrrMiRr0hkFY6tIYY</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 638000000, "_seconds": 1788087134}</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>1788087134638</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L144" t="n">
+        <v>80</v>
+      </c>
+      <c r="M144" t="b">
+        <v>0</v>
+      </c>
+      <c r="N144" t="n">
+        <v>336</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Lactic Acid</t>
+        </is>
+      </c>
+      <c r="Q144" t="b">
+        <v>0</v>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>Water Agent</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>Mash</t>
+        </is>
+      </c>
+      <c r="U144" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y144" t="inlineStr"/>
+      <c r="Z144" t="inlineStr"/>
+      <c r="AA144" t="inlineStr"/>
+      <c r="AB144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 227000000, "_seconds": 1714216066}</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>default-6bc446</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>DtZ4WaKJ79LUfugEJi3A4PwhoDqCzG</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 940000000, "_seconds": 1721546982}</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>1721546982940</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>2</v>
+      </c>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="b">
+        <v>0</v>
+      </c>
+      <c r="N145" t="n">
+        <v>-5</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Biofine Clear</t>
+        </is>
+      </c>
+      <c r="P145" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q145" t="b">
+        <v>1</v>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Fining</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr"/>
+      <c r="Y145" t="inlineStr"/>
+      <c r="Z145" t="inlineStr"/>
+      <c r="AA145" t="inlineStr"/>
+      <c r="AB145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 312000000, "_seconds": 1697269078}</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>default-yn1j28sf</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>5dwZuz6McgWsQTyWei8G44K5IFAD5I</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 144000000, "_seconds": 1723974354}</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>1723974354144</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>2.10.6</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>2</v>
+      </c>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="b">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>-19</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Yeast Nutrients</t>
+        </is>
+      </c>
+      <c r="P146" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q146" t="b">
+        <v>0</v>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr"/>
+      <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr"/>
+      <c r="AB146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>3IHDxeB1SX3QaLERATIxYhFsnmvLZZ</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Old English Summer Stout</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 320000000, "_seconds": 1787845020}</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>FxymQbqWfYaVaT8ypqgApwGcTjOAXm</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>8ohTm584SLfO1z9IbILXf1d0nQqtl4</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>{"_nanoseconds": 14000000, "_seconds": 1788116824}</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>1788116824014</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>1</v>
+      </c>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="b">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>ISY Enhabce</t>
+        </is>
+      </c>
+      <c r="P147" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Boil</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+      <c r="AB147" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB140"/>
+  <autoFilter ref="A1:AB147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>